<commit_message>
Pushing last weeks notebook
</commit_message>
<xml_diff>
--- a/STM.NoiseMethodComp.xlsx
+++ b/STM.NoiseMethodComp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charlesh/Documents/Codes/OBS_Methods/NOISE/ATACR_HPS_Comp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E271BC7-4960-5A40-A509-F4774B5858EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DDEC1EA-D92B-5140-A0D0-04DB3F4818ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{2D23EB00-7FB2-7344-A3A8-C5901D65A225}"/>
   </bookViews>
@@ -1062,22 +1062,43 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1101,6 +1122,9 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1110,19 +1134,19 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1142,30 +1166,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1523,52 +1523,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="83"/>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="82"/>
+      <c r="A1" s="56"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="55"/>
     </row>
     <row r="2" spans="1:45" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="83" t="s">
+      <c r="A2" s="56" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="83"/>
-      <c r="C2" s="83"/>
-      <c r="D2" s="83"/>
-      <c r="E2" s="83"/>
-      <c r="F2" s="82"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="55"/>
     </row>
     <row r="3" spans="1:45" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="83"/>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="82"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="55"/>
     </row>
     <row r="4" spans="1:45" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="83" t="s">
+      <c r="A4" s="56" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="83"/>
-      <c r="C4" s="83"/>
-      <c r="D4" s="83"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="82"/>
+      <c r="B4" s="56"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="55"/>
     </row>
     <row r="5" spans="1:45" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="84" t="s">
+      <c r="A5" s="57" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="83"/>
-      <c r="C5" s="83"/>
-      <c r="D5" s="83"/>
-      <c r="E5" s="83"/>
-      <c r="F5" s="82"/>
+      <c r="B5" s="56"/>
+      <c r="C5" s="56"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="56"/>
+      <c r="F5" s="55"/>
     </row>
     <row r="6" spans="1:45" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="23" t="s">
@@ -1589,41 +1589,41 @@
       <c r="F6" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="K6" s="86"/>
-      <c r="L6" s="86"/>
-      <c r="M6" s="86"/>
-      <c r="N6" s="86"/>
-      <c r="O6" s="86"/>
-      <c r="P6" s="86"/>
-      <c r="Q6" s="86"/>
-      <c r="R6" s="86"/>
-      <c r="S6" s="86"/>
-      <c r="T6" s="86"/>
-      <c r="U6" s="86"/>
-      <c r="V6" s="86"/>
-      <c r="W6" s="86"/>
-      <c r="X6" s="86"/>
-      <c r="Y6" s="86"/>
-      <c r="Z6" s="86"/>
-      <c r="AA6" s="86"/>
-      <c r="AB6" s="86"/>
-      <c r="AC6" s="86"/>
-      <c r="AD6" s="86"/>
-      <c r="AE6" s="86"/>
-      <c r="AF6" s="86"/>
-      <c r="AG6" s="86"/>
-      <c r="AH6" s="86"/>
-      <c r="AI6" s="86"/>
-      <c r="AJ6" s="86"/>
-      <c r="AK6" s="86"/>
-      <c r="AL6" s="86"/>
-      <c r="AM6" s="86"/>
-      <c r="AN6" s="86"/>
-      <c r="AO6" s="86"/>
-      <c r="AP6" s="86"/>
-      <c r="AQ6" s="86"/>
-      <c r="AR6" s="86"/>
-      <c r="AS6" s="86"/>
+      <c r="K6" s="59"/>
+      <c r="L6" s="59"/>
+      <c r="M6" s="59"/>
+      <c r="N6" s="59"/>
+      <c r="O6" s="59"/>
+      <c r="P6" s="59"/>
+      <c r="Q6" s="59"/>
+      <c r="R6" s="59"/>
+      <c r="S6" s="59"/>
+      <c r="T6" s="59"/>
+      <c r="U6" s="59"/>
+      <c r="V6" s="59"/>
+      <c r="W6" s="59"/>
+      <c r="X6" s="59"/>
+      <c r="Y6" s="59"/>
+      <c r="Z6" s="59"/>
+      <c r="AA6" s="59"/>
+      <c r="AB6" s="59"/>
+      <c r="AC6" s="59"/>
+      <c r="AD6" s="59"/>
+      <c r="AE6" s="59"/>
+      <c r="AF6" s="59"/>
+      <c r="AG6" s="59"/>
+      <c r="AH6" s="59"/>
+      <c r="AI6" s="59"/>
+      <c r="AJ6" s="59"/>
+      <c r="AK6" s="59"/>
+      <c r="AL6" s="59"/>
+      <c r="AM6" s="59"/>
+      <c r="AN6" s="59"/>
+      <c r="AO6" s="59"/>
+      <c r="AP6" s="59"/>
+      <c r="AQ6" s="59"/>
+      <c r="AR6" s="59"/>
+      <c r="AS6" s="59"/>
     </row>
     <row r="7" spans="1:45" s="2" customFormat="1" ht="10" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="22"/>
@@ -1632,42 +1632,42 @@
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
       <c r="F7" s="22"/>
-      <c r="H7" s="85"/>
-      <c r="K7" s="87"/>
-      <c r="L7" s="87"/>
-      <c r="M7" s="87"/>
-      <c r="N7" s="87"/>
-      <c r="O7" s="87"/>
-      <c r="P7" s="87"/>
-      <c r="Q7" s="87"/>
-      <c r="R7" s="87"/>
-      <c r="S7" s="87"/>
-      <c r="T7" s="87"/>
-      <c r="U7" s="87"/>
-      <c r="V7" s="87"/>
-      <c r="W7" s="87"/>
-      <c r="X7" s="87"/>
-      <c r="Y7" s="87"/>
-      <c r="Z7" s="87"/>
-      <c r="AA7" s="87"/>
-      <c r="AB7" s="87"/>
-      <c r="AC7" s="87"/>
-      <c r="AD7" s="87"/>
-      <c r="AE7" s="87"/>
-      <c r="AF7" s="87"/>
-      <c r="AG7" s="87"/>
-      <c r="AH7" s="87"/>
-      <c r="AI7" s="87"/>
-      <c r="AJ7" s="87"/>
-      <c r="AK7" s="87"/>
-      <c r="AL7" s="87"/>
-      <c r="AM7" s="87"/>
-      <c r="AN7" s="87"/>
-      <c r="AO7" s="87"/>
-      <c r="AP7" s="87"/>
-      <c r="AQ7" s="87"/>
-      <c r="AR7" s="87"/>
-      <c r="AS7" s="87"/>
+      <c r="H7" s="58"/>
+      <c r="K7" s="60"/>
+      <c r="L7" s="60"/>
+      <c r="M7" s="60"/>
+      <c r="N7" s="60"/>
+      <c r="O7" s="60"/>
+      <c r="P7" s="60"/>
+      <c r="Q7" s="60"/>
+      <c r="R7" s="60"/>
+      <c r="S7" s="60"/>
+      <c r="T7" s="60"/>
+      <c r="U7" s="60"/>
+      <c r="V7" s="60"/>
+      <c r="W7" s="60"/>
+      <c r="X7" s="60"/>
+      <c r="Y7" s="60"/>
+      <c r="Z7" s="60"/>
+      <c r="AA7" s="60"/>
+      <c r="AB7" s="60"/>
+      <c r="AC7" s="60"/>
+      <c r="AD7" s="60"/>
+      <c r="AE7" s="60"/>
+      <c r="AF7" s="60"/>
+      <c r="AG7" s="60"/>
+      <c r="AH7" s="60"/>
+      <c r="AI7" s="60"/>
+      <c r="AJ7" s="60"/>
+      <c r="AK7" s="60"/>
+      <c r="AL7" s="60"/>
+      <c r="AM7" s="60"/>
+      <c r="AN7" s="60"/>
+      <c r="AO7" s="60"/>
+      <c r="AP7" s="60"/>
+      <c r="AQ7" s="60"/>
+      <c r="AR7" s="60"/>
+      <c r="AS7" s="60"/>
     </row>
     <row r="8" spans="1:45" s="5" customFormat="1" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
@@ -1678,41 +1678,41 @@
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
-      <c r="K8" s="88"/>
-      <c r="L8" s="88"/>
-      <c r="M8" s="88"/>
-      <c r="N8" s="88"/>
-      <c r="O8" s="88"/>
-      <c r="P8" s="88"/>
-      <c r="Q8" s="88"/>
-      <c r="R8" s="88"/>
-      <c r="S8" s="88"/>
-      <c r="T8" s="88"/>
-      <c r="U8" s="88"/>
-      <c r="V8" s="88"/>
-      <c r="W8" s="88"/>
-      <c r="X8" s="88"/>
-      <c r="Y8" s="88"/>
-      <c r="Z8" s="88"/>
-      <c r="AA8" s="88"/>
-      <c r="AB8" s="88"/>
-      <c r="AC8" s="88"/>
-      <c r="AD8" s="88"/>
-      <c r="AE8" s="88"/>
-      <c r="AF8" s="88"/>
-      <c r="AG8" s="88"/>
-      <c r="AH8" s="88"/>
-      <c r="AI8" s="88"/>
-      <c r="AJ8" s="88"/>
-      <c r="AK8" s="88"/>
-      <c r="AL8" s="88"/>
-      <c r="AM8" s="88"/>
-      <c r="AN8" s="88"/>
-      <c r="AO8" s="88"/>
-      <c r="AP8" s="88"/>
-      <c r="AQ8" s="88"/>
-      <c r="AR8" s="88"/>
-      <c r="AS8" s="88"/>
+      <c r="K8" s="61"/>
+      <c r="L8" s="61"/>
+      <c r="M8" s="61"/>
+      <c r="N8" s="61"/>
+      <c r="O8" s="61"/>
+      <c r="P8" s="61"/>
+      <c r="Q8" s="61"/>
+      <c r="R8" s="61"/>
+      <c r="S8" s="61"/>
+      <c r="T8" s="61"/>
+      <c r="U8" s="61"/>
+      <c r="V8" s="61"/>
+      <c r="W8" s="61"/>
+      <c r="X8" s="61"/>
+      <c r="Y8" s="61"/>
+      <c r="Z8" s="61"/>
+      <c r="AA8" s="61"/>
+      <c r="AB8" s="61"/>
+      <c r="AC8" s="61"/>
+      <c r="AD8" s="61"/>
+      <c r="AE8" s="61"/>
+      <c r="AF8" s="61"/>
+      <c r="AG8" s="61"/>
+      <c r="AH8" s="61"/>
+      <c r="AI8" s="61"/>
+      <c r="AJ8" s="61"/>
+      <c r="AK8" s="61"/>
+      <c r="AL8" s="61"/>
+      <c r="AM8" s="61"/>
+      <c r="AN8" s="61"/>
+      <c r="AO8" s="61"/>
+      <c r="AP8" s="61"/>
+      <c r="AQ8" s="61"/>
+      <c r="AR8" s="61"/>
+      <c r="AS8" s="61"/>
     </row>
     <row r="9" spans="1:45" s="5" customFormat="1" ht="121" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="51" t="s">
@@ -1729,41 +1729,41 @@
       <c r="F9" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="K9" s="88"/>
-      <c r="L9" s="88"/>
-      <c r="M9" s="88"/>
-      <c r="N9" s="88"/>
-      <c r="O9" s="88"/>
-      <c r="P9" s="88"/>
-      <c r="Q9" s="88"/>
-      <c r="R9" s="88"/>
-      <c r="S9" s="88"/>
-      <c r="T9" s="88"/>
-      <c r="U9" s="88"/>
-      <c r="V9" s="88"/>
-      <c r="W9" s="88"/>
-      <c r="X9" s="88"/>
-      <c r="Y9" s="88"/>
-      <c r="Z9" s="88"/>
-      <c r="AA9" s="88"/>
-      <c r="AB9" s="88"/>
-      <c r="AC9" s="88"/>
-      <c r="AD9" s="88"/>
-      <c r="AE9" s="88"/>
-      <c r="AF9" s="88"/>
-      <c r="AG9" s="88"/>
-      <c r="AH9" s="88"/>
-      <c r="AI9" s="88"/>
-      <c r="AJ9" s="88"/>
-      <c r="AK9" s="88"/>
-      <c r="AL9" s="88"/>
-      <c r="AM9" s="88"/>
-      <c r="AN9" s="88"/>
-      <c r="AO9" s="88"/>
-      <c r="AP9" s="88"/>
-      <c r="AQ9" s="88"/>
-      <c r="AR9" s="88"/>
-      <c r="AS9" s="88"/>
+      <c r="K9" s="61"/>
+      <c r="L9" s="61"/>
+      <c r="M9" s="61"/>
+      <c r="N9" s="61"/>
+      <c r="O9" s="61"/>
+      <c r="P9" s="61"/>
+      <c r="Q9" s="61"/>
+      <c r="R9" s="61"/>
+      <c r="S9" s="61"/>
+      <c r="T9" s="61"/>
+      <c r="U9" s="61"/>
+      <c r="V9" s="61"/>
+      <c r="W9" s="61"/>
+      <c r="X9" s="61"/>
+      <c r="Y9" s="61"/>
+      <c r="Z9" s="61"/>
+      <c r="AA9" s="61"/>
+      <c r="AB9" s="61"/>
+      <c r="AC9" s="61"/>
+      <c r="AD9" s="61"/>
+      <c r="AE9" s="61"/>
+      <c r="AF9" s="61"/>
+      <c r="AG9" s="61"/>
+      <c r="AH9" s="61"/>
+      <c r="AI9" s="61"/>
+      <c r="AJ9" s="61"/>
+      <c r="AK9" s="61"/>
+      <c r="AL9" s="61"/>
+      <c r="AM9" s="61"/>
+      <c r="AN9" s="61"/>
+      <c r="AO9" s="61"/>
+      <c r="AP9" s="61"/>
+      <c r="AQ9" s="61"/>
+      <c r="AR9" s="61"/>
+      <c r="AS9" s="61"/>
     </row>
     <row r="10" spans="1:45" s="5" customFormat="1" ht="49" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="52"/>
@@ -1774,86 +1774,86 @@
       <c r="D10" s="20"/>
       <c r="E10" s="20"/>
       <c r="F10" s="20"/>
-      <c r="K10" s="88"/>
-      <c r="L10" s="88"/>
-      <c r="M10" s="88"/>
-      <c r="N10" s="88"/>
-      <c r="O10" s="88"/>
-      <c r="P10" s="88"/>
-      <c r="Q10" s="88"/>
-      <c r="R10" s="88"/>
-      <c r="S10" s="88"/>
-      <c r="T10" s="88"/>
-      <c r="U10" s="88"/>
-      <c r="V10" s="88"/>
-      <c r="W10" s="88"/>
-      <c r="X10" s="88"/>
-      <c r="Y10" s="88"/>
-      <c r="Z10" s="88"/>
-      <c r="AA10" s="88"/>
-      <c r="AB10" s="88"/>
-      <c r="AC10" s="88"/>
-      <c r="AD10" s="88"/>
-      <c r="AE10" s="88"/>
-      <c r="AF10" s="88"/>
-      <c r="AG10" s="88"/>
-      <c r="AH10" s="88"/>
-      <c r="AI10" s="88"/>
-      <c r="AJ10" s="88"/>
-      <c r="AK10" s="88"/>
-      <c r="AL10" s="88"/>
-      <c r="AM10" s="88"/>
-      <c r="AN10" s="88"/>
-      <c r="AO10" s="88"/>
-      <c r="AP10" s="88"/>
-      <c r="AQ10" s="88"/>
-      <c r="AR10" s="88"/>
-      <c r="AS10" s="88"/>
+      <c r="K10" s="61"/>
+      <c r="L10" s="61"/>
+      <c r="M10" s="61"/>
+      <c r="N10" s="61"/>
+      <c r="O10" s="61"/>
+      <c r="P10" s="61"/>
+      <c r="Q10" s="61"/>
+      <c r="R10" s="61"/>
+      <c r="S10" s="61"/>
+      <c r="T10" s="61"/>
+      <c r="U10" s="61"/>
+      <c r="V10" s="61"/>
+      <c r="W10" s="61"/>
+      <c r="X10" s="61"/>
+      <c r="Y10" s="61"/>
+      <c r="Z10" s="61"/>
+      <c r="AA10" s="61"/>
+      <c r="AB10" s="61"/>
+      <c r="AC10" s="61"/>
+      <c r="AD10" s="61"/>
+      <c r="AE10" s="61"/>
+      <c r="AF10" s="61"/>
+      <c r="AG10" s="61"/>
+      <c r="AH10" s="61"/>
+      <c r="AI10" s="61"/>
+      <c r="AJ10" s="61"/>
+      <c r="AK10" s="61"/>
+      <c r="AL10" s="61"/>
+      <c r="AM10" s="61"/>
+      <c r="AN10" s="61"/>
+      <c r="AO10" s="61"/>
+      <c r="AP10" s="61"/>
+      <c r="AQ10" s="61"/>
+      <c r="AR10" s="61"/>
+      <c r="AS10" s="61"/>
     </row>
     <row r="11" spans="1:45" s="5" customFormat="1" ht="23" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="52"/>
       <c r="B11" s="48"/>
       <c r="C11" s="41"/>
-      <c r="D11" s="55" t="s">
+      <c r="D11" s="79" t="s">
         <v>37</v>
       </c>
-      <c r="E11" s="55"/>
-      <c r="F11" s="56"/>
-      <c r="K11" s="88"/>
-      <c r="L11" s="88"/>
-      <c r="M11" s="88"/>
-      <c r="N11" s="88"/>
-      <c r="O11" s="88"/>
-      <c r="P11" s="88"/>
-      <c r="Q11" s="88"/>
-      <c r="R11" s="88"/>
-      <c r="S11" s="88"/>
-      <c r="T11" s="88"/>
-      <c r="U11" s="88"/>
-      <c r="V11" s="88"/>
-      <c r="W11" s="88"/>
-      <c r="X11" s="88"/>
-      <c r="Y11" s="88"/>
-      <c r="Z11" s="88"/>
-      <c r="AA11" s="88"/>
-      <c r="AB11" s="88"/>
-      <c r="AC11" s="88"/>
-      <c r="AD11" s="88"/>
-      <c r="AE11" s="88"/>
-      <c r="AF11" s="88"/>
-      <c r="AG11" s="88"/>
-      <c r="AH11" s="88"/>
-      <c r="AI11" s="88"/>
-      <c r="AJ11" s="88"/>
-      <c r="AK11" s="88"/>
-      <c r="AL11" s="88"/>
-      <c r="AM11" s="88"/>
-      <c r="AN11" s="88"/>
-      <c r="AO11" s="88"/>
-      <c r="AP11" s="88"/>
-      <c r="AQ11" s="88"/>
-      <c r="AR11" s="88"/>
-      <c r="AS11" s="88"/>
+      <c r="E11" s="79"/>
+      <c r="F11" s="80"/>
+      <c r="K11" s="61"/>
+      <c r="L11" s="61"/>
+      <c r="M11" s="61"/>
+      <c r="N11" s="61"/>
+      <c r="O11" s="61"/>
+      <c r="P11" s="61"/>
+      <c r="Q11" s="61"/>
+      <c r="R11" s="61"/>
+      <c r="S11" s="61"/>
+      <c r="T11" s="61"/>
+      <c r="U11" s="61"/>
+      <c r="V11" s="61"/>
+      <c r="W11" s="61"/>
+      <c r="X11" s="61"/>
+      <c r="Y11" s="61"/>
+      <c r="Z11" s="61"/>
+      <c r="AA11" s="61"/>
+      <c r="AB11" s="61"/>
+      <c r="AC11" s="61"/>
+      <c r="AD11" s="61"/>
+      <c r="AE11" s="61"/>
+      <c r="AF11" s="61"/>
+      <c r="AG11" s="61"/>
+      <c r="AH11" s="61"/>
+      <c r="AI11" s="61"/>
+      <c r="AJ11" s="61"/>
+      <c r="AK11" s="61"/>
+      <c r="AL11" s="61"/>
+      <c r="AM11" s="61"/>
+      <c r="AN11" s="61"/>
+      <c r="AO11" s="61"/>
+      <c r="AP11" s="61"/>
+      <c r="AQ11" s="61"/>
+      <c r="AR11" s="61"/>
+      <c r="AS11" s="61"/>
     </row>
     <row r="12" spans="1:45" s="5" customFormat="1" ht="210" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="52"/>
@@ -1868,86 +1868,86 @@
       <c r="F12" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="K12" s="88"/>
-      <c r="L12" s="88"/>
-      <c r="M12" s="88"/>
-      <c r="N12" s="88"/>
-      <c r="O12" s="88"/>
-      <c r="P12" s="88"/>
-      <c r="Q12" s="88"/>
-      <c r="R12" s="88"/>
-      <c r="S12" s="88"/>
-      <c r="T12" s="88"/>
-      <c r="U12" s="88"/>
-      <c r="V12" s="88"/>
-      <c r="W12" s="88"/>
-      <c r="X12" s="88"/>
-      <c r="Y12" s="88"/>
-      <c r="Z12" s="88"/>
-      <c r="AA12" s="88"/>
-      <c r="AB12" s="88"/>
-      <c r="AC12" s="88"/>
-      <c r="AD12" s="88"/>
-      <c r="AE12" s="88"/>
-      <c r="AF12" s="88"/>
-      <c r="AG12" s="88"/>
-      <c r="AH12" s="88"/>
-      <c r="AI12" s="88"/>
-      <c r="AJ12" s="88"/>
-      <c r="AK12" s="88"/>
-      <c r="AL12" s="88"/>
-      <c r="AM12" s="88"/>
-      <c r="AN12" s="88"/>
-      <c r="AO12" s="88"/>
-      <c r="AP12" s="88"/>
-      <c r="AQ12" s="88"/>
-      <c r="AR12" s="88"/>
-      <c r="AS12" s="88"/>
+      <c r="K12" s="61"/>
+      <c r="L12" s="61"/>
+      <c r="M12" s="61"/>
+      <c r="N12" s="61"/>
+      <c r="O12" s="61"/>
+      <c r="P12" s="61"/>
+      <c r="Q12" s="61"/>
+      <c r="R12" s="61"/>
+      <c r="S12" s="61"/>
+      <c r="T12" s="61"/>
+      <c r="U12" s="61"/>
+      <c r="V12" s="61"/>
+      <c r="W12" s="61"/>
+      <c r="X12" s="61"/>
+      <c r="Y12" s="61"/>
+      <c r="Z12" s="61"/>
+      <c r="AA12" s="61"/>
+      <c r="AB12" s="61"/>
+      <c r="AC12" s="61"/>
+      <c r="AD12" s="61"/>
+      <c r="AE12" s="61"/>
+      <c r="AF12" s="61"/>
+      <c r="AG12" s="61"/>
+      <c r="AH12" s="61"/>
+      <c r="AI12" s="61"/>
+      <c r="AJ12" s="61"/>
+      <c r="AK12" s="61"/>
+      <c r="AL12" s="61"/>
+      <c r="AM12" s="61"/>
+      <c r="AN12" s="61"/>
+      <c r="AO12" s="61"/>
+      <c r="AP12" s="61"/>
+      <c r="AQ12" s="61"/>
+      <c r="AR12" s="61"/>
+      <c r="AS12" s="61"/>
     </row>
     <row r="13" spans="1:45" s="5" customFormat="1" ht="56" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="52"/>
-      <c r="B13" s="76" t="s">
+      <c r="B13" s="84" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="77"/>
-      <c r="D13" s="77"/>
-      <c r="E13" s="77"/>
-      <c r="F13" s="78"/>
-      <c r="K13" s="88"/>
-      <c r="L13" s="88"/>
-      <c r="M13" s="88"/>
-      <c r="N13" s="88"/>
-      <c r="O13" s="88"/>
-      <c r="P13" s="88"/>
-      <c r="Q13" s="88"/>
-      <c r="R13" s="88"/>
-      <c r="S13" s="88"/>
-      <c r="T13" s="88"/>
-      <c r="U13" s="88"/>
-      <c r="V13" s="88"/>
-      <c r="W13" s="88"/>
-      <c r="X13" s="88"/>
-      <c r="Y13" s="88"/>
-      <c r="Z13" s="88"/>
-      <c r="AA13" s="88"/>
-      <c r="AB13" s="88"/>
-      <c r="AC13" s="88"/>
-      <c r="AD13" s="88"/>
-      <c r="AE13" s="88"/>
-      <c r="AF13" s="88"/>
-      <c r="AG13" s="88"/>
-      <c r="AH13" s="88"/>
-      <c r="AI13" s="88"/>
-      <c r="AJ13" s="88"/>
-      <c r="AK13" s="88"/>
-      <c r="AL13" s="88"/>
-      <c r="AM13" s="88"/>
-      <c r="AN13" s="88"/>
-      <c r="AO13" s="88"/>
-      <c r="AP13" s="88"/>
-      <c r="AQ13" s="88"/>
-      <c r="AR13" s="88"/>
-      <c r="AS13" s="88"/>
+      <c r="C13" s="85"/>
+      <c r="D13" s="85"/>
+      <c r="E13" s="85"/>
+      <c r="F13" s="86"/>
+      <c r="K13" s="61"/>
+      <c r="L13" s="61"/>
+      <c r="M13" s="61"/>
+      <c r="N13" s="61"/>
+      <c r="O13" s="61"/>
+      <c r="P13" s="61"/>
+      <c r="Q13" s="61"/>
+      <c r="R13" s="61"/>
+      <c r="S13" s="61"/>
+      <c r="T13" s="61"/>
+      <c r="U13" s="61"/>
+      <c r="V13" s="61"/>
+      <c r="W13" s="61"/>
+      <c r="X13" s="61"/>
+      <c r="Y13" s="61"/>
+      <c r="Z13" s="61"/>
+      <c r="AA13" s="61"/>
+      <c r="AB13" s="61"/>
+      <c r="AC13" s="61"/>
+      <c r="AD13" s="61"/>
+      <c r="AE13" s="61"/>
+      <c r="AF13" s="61"/>
+      <c r="AG13" s="61"/>
+      <c r="AH13" s="61"/>
+      <c r="AI13" s="61"/>
+      <c r="AJ13" s="61"/>
+      <c r="AK13" s="61"/>
+      <c r="AL13" s="61"/>
+      <c r="AM13" s="61"/>
+      <c r="AN13" s="61"/>
+      <c r="AO13" s="61"/>
+      <c r="AP13" s="61"/>
+      <c r="AQ13" s="61"/>
+      <c r="AR13" s="61"/>
+      <c r="AS13" s="61"/>
     </row>
     <row r="14" spans="1:45" s="8" customFormat="1" ht="121" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="53"/>
@@ -1955,47 +1955,47 @@
       <c r="C14" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="79" t="s">
+      <c r="D14" s="87" t="s">
         <v>36</v>
       </c>
-      <c r="E14" s="80"/>
-      <c r="F14" s="81"/>
+      <c r="E14" s="88"/>
+      <c r="F14" s="89"/>
       <c r="I14" s="5"/>
-      <c r="K14" s="89"/>
-      <c r="L14" s="89"/>
-      <c r="M14" s="89"/>
-      <c r="N14" s="89"/>
-      <c r="O14" s="89"/>
-      <c r="P14" s="89"/>
-      <c r="Q14" s="89"/>
-      <c r="R14" s="89"/>
-      <c r="S14" s="89"/>
-      <c r="T14" s="89"/>
-      <c r="U14" s="89"/>
-      <c r="V14" s="89"/>
-      <c r="W14" s="89"/>
-      <c r="X14" s="89"/>
-      <c r="Y14" s="89"/>
-      <c r="Z14" s="89"/>
-      <c r="AA14" s="89"/>
-      <c r="AB14" s="89"/>
-      <c r="AC14" s="89"/>
-      <c r="AD14" s="89"/>
-      <c r="AE14" s="89"/>
-      <c r="AF14" s="89"/>
-      <c r="AG14" s="89"/>
-      <c r="AH14" s="89"/>
-      <c r="AI14" s="89"/>
-      <c r="AJ14" s="89"/>
-      <c r="AK14" s="89"/>
-      <c r="AL14" s="89"/>
-      <c r="AM14" s="89"/>
-      <c r="AN14" s="89"/>
-      <c r="AO14" s="89"/>
-      <c r="AP14" s="89"/>
-      <c r="AQ14" s="89"/>
-      <c r="AR14" s="89"/>
-      <c r="AS14" s="89"/>
+      <c r="K14" s="62"/>
+      <c r="L14" s="62"/>
+      <c r="M14" s="62"/>
+      <c r="N14" s="62"/>
+      <c r="O14" s="62"/>
+      <c r="P14" s="62"/>
+      <c r="Q14" s="62"/>
+      <c r="R14" s="62"/>
+      <c r="S14" s="62"/>
+      <c r="T14" s="62"/>
+      <c r="U14" s="62"/>
+      <c r="V14" s="62"/>
+      <c r="W14" s="62"/>
+      <c r="X14" s="62"/>
+      <c r="Y14" s="62"/>
+      <c r="Z14" s="62"/>
+      <c r="AA14" s="62"/>
+      <c r="AB14" s="62"/>
+      <c r="AC14" s="62"/>
+      <c r="AD14" s="62"/>
+      <c r="AE14" s="62"/>
+      <c r="AF14" s="62"/>
+      <c r="AG14" s="62"/>
+      <c r="AH14" s="62"/>
+      <c r="AI14" s="62"/>
+      <c r="AJ14" s="62"/>
+      <c r="AK14" s="62"/>
+      <c r="AL14" s="62"/>
+      <c r="AM14" s="62"/>
+      <c r="AN14" s="62"/>
+      <c r="AO14" s="62"/>
+      <c r="AP14" s="62"/>
+      <c r="AQ14" s="62"/>
+      <c r="AR14" s="62"/>
+      <c r="AS14" s="62"/>
     </row>
     <row r="15" spans="1:45" s="8" customFormat="1" ht="70" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="53"/>
@@ -2007,777 +2007,777 @@
         <v>28</v>
       </c>
       <c r="I15" s="5"/>
-      <c r="K15" s="89"/>
-      <c r="L15" s="89"/>
-      <c r="M15" s="89"/>
-      <c r="N15" s="89"/>
-      <c r="O15" s="89"/>
-      <c r="P15" s="89"/>
-      <c r="Q15" s="89"/>
-      <c r="R15" s="89"/>
-      <c r="S15" s="89"/>
-      <c r="T15" s="89"/>
-      <c r="U15" s="89"/>
-      <c r="V15" s="89"/>
-      <c r="W15" s="89"/>
-      <c r="X15" s="89"/>
-      <c r="Y15" s="89"/>
-      <c r="Z15" s="89"/>
-      <c r="AA15" s="89"/>
-      <c r="AB15" s="89"/>
-      <c r="AC15" s="89"/>
-      <c r="AD15" s="89"/>
-      <c r="AE15" s="89"/>
-      <c r="AF15" s="89"/>
-      <c r="AG15" s="89"/>
-      <c r="AH15" s="89"/>
-      <c r="AI15" s="89"/>
-      <c r="AJ15" s="89"/>
-      <c r="AK15" s="89"/>
-      <c r="AL15" s="89"/>
-      <c r="AM15" s="89"/>
-      <c r="AN15" s="89"/>
-      <c r="AO15" s="89"/>
-      <c r="AP15" s="89"/>
-      <c r="AQ15" s="89"/>
-      <c r="AR15" s="89"/>
-      <c r="AS15" s="89"/>
+      <c r="K15" s="62"/>
+      <c r="L15" s="62"/>
+      <c r="M15" s="62"/>
+      <c r="N15" s="62"/>
+      <c r="O15" s="62"/>
+      <c r="P15" s="62"/>
+      <c r="Q15" s="62"/>
+      <c r="R15" s="62"/>
+      <c r="S15" s="62"/>
+      <c r="T15" s="62"/>
+      <c r="U15" s="62"/>
+      <c r="V15" s="62"/>
+      <c r="W15" s="62"/>
+      <c r="X15" s="62"/>
+      <c r="Y15" s="62"/>
+      <c r="Z15" s="62"/>
+      <c r="AA15" s="62"/>
+      <c r="AB15" s="62"/>
+      <c r="AC15" s="62"/>
+      <c r="AD15" s="62"/>
+      <c r="AE15" s="62"/>
+      <c r="AF15" s="62"/>
+      <c r="AG15" s="62"/>
+      <c r="AH15" s="62"/>
+      <c r="AI15" s="62"/>
+      <c r="AJ15" s="62"/>
+      <c r="AK15" s="62"/>
+      <c r="AL15" s="62"/>
+      <c r="AM15" s="62"/>
+      <c r="AN15" s="62"/>
+      <c r="AO15" s="62"/>
+      <c r="AP15" s="62"/>
+      <c r="AQ15" s="62"/>
+      <c r="AR15" s="62"/>
+      <c r="AS15" s="62"/>
     </row>
     <row r="16" spans="1:45" s="8" customFormat="1" ht="23" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="53"/>
       <c r="B16" s="28"/>
       <c r="C16" s="44"/>
-      <c r="D16" s="57" t="s">
+      <c r="D16" s="81" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="57"/>
-      <c r="F16" s="58"/>
-      <c r="K16" s="89"/>
-      <c r="L16" s="89"/>
-      <c r="M16" s="89"/>
-      <c r="N16" s="89"/>
-      <c r="O16" s="89"/>
-      <c r="P16" s="89"/>
-      <c r="Q16" s="89"/>
-      <c r="R16" s="89"/>
-      <c r="S16" s="89"/>
-      <c r="T16" s="89"/>
-      <c r="U16" s="89"/>
-      <c r="V16" s="89"/>
-      <c r="W16" s="89"/>
-      <c r="X16" s="89"/>
-      <c r="Y16" s="89"/>
-      <c r="Z16" s="89"/>
-      <c r="AA16" s="89"/>
-      <c r="AB16" s="89"/>
-      <c r="AC16" s="89"/>
-      <c r="AD16" s="89"/>
-      <c r="AE16" s="89"/>
-      <c r="AF16" s="89"/>
-      <c r="AG16" s="89"/>
-      <c r="AH16" s="89"/>
-      <c r="AI16" s="89"/>
-      <c r="AJ16" s="89"/>
-      <c r="AK16" s="89"/>
-      <c r="AL16" s="89"/>
-      <c r="AM16" s="89"/>
-      <c r="AN16" s="89"/>
-      <c r="AO16" s="89"/>
-      <c r="AP16" s="89"/>
-      <c r="AQ16" s="89"/>
-      <c r="AR16" s="89"/>
-      <c r="AS16" s="89"/>
+      <c r="E16" s="81"/>
+      <c r="F16" s="82"/>
+      <c r="K16" s="62"/>
+      <c r="L16" s="62"/>
+      <c r="M16" s="62"/>
+      <c r="N16" s="62"/>
+      <c r="O16" s="62"/>
+      <c r="P16" s="62"/>
+      <c r="Q16" s="62"/>
+      <c r="R16" s="62"/>
+      <c r="S16" s="62"/>
+      <c r="T16" s="62"/>
+      <c r="U16" s="62"/>
+      <c r="V16" s="62"/>
+      <c r="W16" s="62"/>
+      <c r="X16" s="62"/>
+      <c r="Y16" s="62"/>
+      <c r="Z16" s="62"/>
+      <c r="AA16" s="62"/>
+      <c r="AB16" s="62"/>
+      <c r="AC16" s="62"/>
+      <c r="AD16" s="62"/>
+      <c r="AE16" s="62"/>
+      <c r="AF16" s="62"/>
+      <c r="AG16" s="62"/>
+      <c r="AH16" s="62"/>
+      <c r="AI16" s="62"/>
+      <c r="AJ16" s="62"/>
+      <c r="AK16" s="62"/>
+      <c r="AL16" s="62"/>
+      <c r="AM16" s="62"/>
+      <c r="AN16" s="62"/>
+      <c r="AO16" s="62"/>
+      <c r="AP16" s="62"/>
+      <c r="AQ16" s="62"/>
+      <c r="AR16" s="62"/>
+      <c r="AS16" s="62"/>
     </row>
     <row r="17" spans="1:45" s="8" customFormat="1" ht="55" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="53"/>
       <c r="B17" s="28"/>
       <c r="C17" s="44"/>
-      <c r="D17" s="59" t="s">
+      <c r="D17" s="83" t="s">
         <v>30</v>
       </c>
-      <c r="E17" s="59"/>
-      <c r="F17" s="59"/>
-      <c r="K17" s="89"/>
-      <c r="L17" s="89"/>
-      <c r="M17" s="89"/>
-      <c r="N17" s="89"/>
-      <c r="O17" s="89"/>
-      <c r="P17" s="89"/>
-      <c r="Q17" s="89"/>
-      <c r="R17" s="89"/>
-      <c r="S17" s="89"/>
-      <c r="T17" s="89"/>
-      <c r="U17" s="89"/>
-      <c r="V17" s="89"/>
-      <c r="W17" s="89"/>
-      <c r="X17" s="89"/>
-      <c r="Y17" s="89"/>
-      <c r="Z17" s="89"/>
-      <c r="AA17" s="89"/>
-      <c r="AB17" s="89"/>
-      <c r="AC17" s="89"/>
-      <c r="AD17" s="89"/>
-      <c r="AE17" s="89"/>
-      <c r="AF17" s="89"/>
-      <c r="AG17" s="89"/>
-      <c r="AH17" s="89"/>
-      <c r="AI17" s="89"/>
-      <c r="AJ17" s="89"/>
-      <c r="AK17" s="89"/>
-      <c r="AL17" s="89"/>
-      <c r="AM17" s="89"/>
-      <c r="AN17" s="89"/>
-      <c r="AO17" s="89"/>
-      <c r="AP17" s="89"/>
-      <c r="AQ17" s="89"/>
-      <c r="AR17" s="89"/>
-      <c r="AS17" s="89"/>
+      <c r="E17" s="83"/>
+      <c r="F17" s="83"/>
+      <c r="K17" s="62"/>
+      <c r="L17" s="62"/>
+      <c r="M17" s="62"/>
+      <c r="N17" s="62"/>
+      <c r="O17" s="62"/>
+      <c r="P17" s="62"/>
+      <c r="Q17" s="62"/>
+      <c r="R17" s="62"/>
+      <c r="S17" s="62"/>
+      <c r="T17" s="62"/>
+      <c r="U17" s="62"/>
+      <c r="V17" s="62"/>
+      <c r="W17" s="62"/>
+      <c r="X17" s="62"/>
+      <c r="Y17" s="62"/>
+      <c r="Z17" s="62"/>
+      <c r="AA17" s="62"/>
+      <c r="AB17" s="62"/>
+      <c r="AC17" s="62"/>
+      <c r="AD17" s="62"/>
+      <c r="AE17" s="62"/>
+      <c r="AF17" s="62"/>
+      <c r="AG17" s="62"/>
+      <c r="AH17" s="62"/>
+      <c r="AI17" s="62"/>
+      <c r="AJ17" s="62"/>
+      <c r="AK17" s="62"/>
+      <c r="AL17" s="62"/>
+      <c r="AM17" s="62"/>
+      <c r="AN17" s="62"/>
+      <c r="AO17" s="62"/>
+      <c r="AP17" s="62"/>
+      <c r="AQ17" s="62"/>
+      <c r="AR17" s="62"/>
+      <c r="AS17" s="62"/>
     </row>
     <row r="18" spans="1:45" s="8" customFormat="1" ht="37" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="53"/>
       <c r="B18" s="28"/>
       <c r="C18" s="44"/>
-      <c r="D18" s="60" t="s">
+      <c r="D18" s="75" t="s">
         <v>31</v>
       </c>
-      <c r="E18" s="63" t="s">
+      <c r="E18" s="70" t="s">
         <v>25</v>
       </c>
-      <c r="F18" s="64"/>
-      <c r="K18" s="89"/>
-      <c r="L18" s="89"/>
-      <c r="M18" s="89"/>
-      <c r="N18" s="89"/>
-      <c r="O18" s="89"/>
-      <c r="P18" s="89"/>
-      <c r="Q18" s="89"/>
-      <c r="R18" s="89"/>
-      <c r="S18" s="89"/>
-      <c r="T18" s="89"/>
-      <c r="U18" s="89"/>
-      <c r="V18" s="89"/>
-      <c r="W18" s="89"/>
-      <c r="X18" s="89"/>
-      <c r="Y18" s="89"/>
-      <c r="Z18" s="89"/>
-      <c r="AA18" s="89"/>
-      <c r="AB18" s="89"/>
-      <c r="AC18" s="89"/>
-      <c r="AD18" s="89"/>
-      <c r="AE18" s="89"/>
-      <c r="AF18" s="89"/>
-      <c r="AG18" s="89"/>
-      <c r="AH18" s="89"/>
-      <c r="AI18" s="89"/>
-      <c r="AJ18" s="89"/>
-      <c r="AK18" s="89"/>
-      <c r="AL18" s="89"/>
-      <c r="AM18" s="89"/>
-      <c r="AN18" s="89"/>
-      <c r="AO18" s="89"/>
-      <c r="AP18" s="89"/>
-      <c r="AQ18" s="89"/>
-      <c r="AR18" s="89"/>
-      <c r="AS18" s="89"/>
+      <c r="F18" s="71"/>
+      <c r="K18" s="62"/>
+      <c r="L18" s="62"/>
+      <c r="M18" s="62"/>
+      <c r="N18" s="62"/>
+      <c r="O18" s="62"/>
+      <c r="P18" s="62"/>
+      <c r="Q18" s="62"/>
+      <c r="R18" s="62"/>
+      <c r="S18" s="62"/>
+      <c r="T18" s="62"/>
+      <c r="U18" s="62"/>
+      <c r="V18" s="62"/>
+      <c r="W18" s="62"/>
+      <c r="X18" s="62"/>
+      <c r="Y18" s="62"/>
+      <c r="Z18" s="62"/>
+      <c r="AA18" s="62"/>
+      <c r="AB18" s="62"/>
+      <c r="AC18" s="62"/>
+      <c r="AD18" s="62"/>
+      <c r="AE18" s="62"/>
+      <c r="AF18" s="62"/>
+      <c r="AG18" s="62"/>
+      <c r="AH18" s="62"/>
+      <c r="AI18" s="62"/>
+      <c r="AJ18" s="62"/>
+      <c r="AK18" s="62"/>
+      <c r="AL18" s="62"/>
+      <c r="AM18" s="62"/>
+      <c r="AN18" s="62"/>
+      <c r="AO18" s="62"/>
+      <c r="AP18" s="62"/>
+      <c r="AQ18" s="62"/>
+      <c r="AR18" s="62"/>
+      <c r="AS18" s="62"/>
     </row>
     <row r="19" spans="1:45" s="8" customFormat="1" ht="121" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="53"/>
       <c r="B19" s="28"/>
       <c r="C19" s="44"/>
-      <c r="D19" s="60"/>
+      <c r="D19" s="75"/>
       <c r="E19" s="38" t="s">
         <v>29</v>
       </c>
       <c r="F19" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="K19" s="89"/>
-      <c r="L19" s="89"/>
-      <c r="M19" s="89"/>
-      <c r="N19" s="89"/>
-      <c r="O19" s="89"/>
-      <c r="P19" s="89"/>
-      <c r="Q19" s="89"/>
-      <c r="R19" s="89"/>
-      <c r="S19" s="89"/>
-      <c r="T19" s="89"/>
-      <c r="U19" s="89"/>
-      <c r="V19" s="89"/>
-      <c r="W19" s="89"/>
-      <c r="X19" s="89"/>
-      <c r="Y19" s="89"/>
-      <c r="Z19" s="89"/>
-      <c r="AA19" s="89"/>
-      <c r="AB19" s="89"/>
-      <c r="AC19" s="89"/>
-      <c r="AD19" s="89"/>
-      <c r="AE19" s="89"/>
-      <c r="AF19" s="89"/>
-      <c r="AG19" s="89"/>
-      <c r="AH19" s="89"/>
-      <c r="AI19" s="89"/>
-      <c r="AJ19" s="89"/>
-      <c r="AK19" s="89"/>
-      <c r="AL19" s="89"/>
-      <c r="AM19" s="89"/>
-      <c r="AN19" s="89"/>
-      <c r="AO19" s="89"/>
-      <c r="AP19" s="89"/>
-      <c r="AQ19" s="89"/>
-      <c r="AR19" s="89"/>
-      <c r="AS19" s="89"/>
+      <c r="K19" s="62"/>
+      <c r="L19" s="62"/>
+      <c r="M19" s="62"/>
+      <c r="N19" s="62"/>
+      <c r="O19" s="62"/>
+      <c r="P19" s="62"/>
+      <c r="Q19" s="62"/>
+      <c r="R19" s="62"/>
+      <c r="S19" s="62"/>
+      <c r="T19" s="62"/>
+      <c r="U19" s="62"/>
+      <c r="V19" s="62"/>
+      <c r="W19" s="62"/>
+      <c r="X19" s="62"/>
+      <c r="Y19" s="62"/>
+      <c r="Z19" s="62"/>
+      <c r="AA19" s="62"/>
+      <c r="AB19" s="62"/>
+      <c r="AC19" s="62"/>
+      <c r="AD19" s="62"/>
+      <c r="AE19" s="62"/>
+      <c r="AF19" s="62"/>
+      <c r="AG19" s="62"/>
+      <c r="AH19" s="62"/>
+      <c r="AI19" s="62"/>
+      <c r="AJ19" s="62"/>
+      <c r="AK19" s="62"/>
+      <c r="AL19" s="62"/>
+      <c r="AM19" s="62"/>
+      <c r="AN19" s="62"/>
+      <c r="AO19" s="62"/>
+      <c r="AP19" s="62"/>
+      <c r="AQ19" s="62"/>
+      <c r="AR19" s="62"/>
+      <c r="AS19" s="62"/>
     </row>
     <row r="20" spans="1:45" s="8" customFormat="1" ht="38" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="53"/>
       <c r="B20" s="28"/>
       <c r="C20" s="44"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="61" t="s">
+      <c r="D20" s="75"/>
+      <c r="E20" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="F20" s="62"/>
-      <c r="K20" s="89"/>
-      <c r="L20" s="89"/>
-      <c r="M20" s="89"/>
-      <c r="N20" s="89"/>
-      <c r="O20" s="89"/>
-      <c r="P20" s="89"/>
-      <c r="Q20" s="89"/>
-      <c r="R20" s="89"/>
-      <c r="S20" s="89"/>
-      <c r="T20" s="89"/>
-      <c r="U20" s="89"/>
-      <c r="V20" s="89"/>
-      <c r="W20" s="89"/>
-      <c r="X20" s="89"/>
-      <c r="Y20" s="89"/>
-      <c r="Z20" s="89"/>
-      <c r="AA20" s="89"/>
-      <c r="AB20" s="89"/>
-      <c r="AC20" s="89"/>
-      <c r="AD20" s="89"/>
-      <c r="AE20" s="89"/>
-      <c r="AF20" s="89"/>
-      <c r="AG20" s="89"/>
-      <c r="AH20" s="89"/>
-      <c r="AI20" s="89"/>
-      <c r="AJ20" s="89"/>
-      <c r="AK20" s="89"/>
-      <c r="AL20" s="89"/>
-      <c r="AM20" s="89"/>
-      <c r="AN20" s="89"/>
-      <c r="AO20" s="89"/>
-      <c r="AP20" s="89"/>
-      <c r="AQ20" s="89"/>
-      <c r="AR20" s="89"/>
-      <c r="AS20" s="89"/>
+      <c r="F20" s="69"/>
+      <c r="K20" s="62"/>
+      <c r="L20" s="62"/>
+      <c r="M20" s="62"/>
+      <c r="N20" s="62"/>
+      <c r="O20" s="62"/>
+      <c r="P20" s="62"/>
+      <c r="Q20" s="62"/>
+      <c r="R20" s="62"/>
+      <c r="S20" s="62"/>
+      <c r="T20" s="62"/>
+      <c r="U20" s="62"/>
+      <c r="V20" s="62"/>
+      <c r="W20" s="62"/>
+      <c r="X20" s="62"/>
+      <c r="Y20" s="62"/>
+      <c r="Z20" s="62"/>
+      <c r="AA20" s="62"/>
+      <c r="AB20" s="62"/>
+      <c r="AC20" s="62"/>
+      <c r="AD20" s="62"/>
+      <c r="AE20" s="62"/>
+      <c r="AF20" s="62"/>
+      <c r="AG20" s="62"/>
+      <c r="AH20" s="62"/>
+      <c r="AI20" s="62"/>
+      <c r="AJ20" s="62"/>
+      <c r="AK20" s="62"/>
+      <c r="AL20" s="62"/>
+      <c r="AM20" s="62"/>
+      <c r="AN20" s="62"/>
+      <c r="AO20" s="62"/>
+      <c r="AP20" s="62"/>
+      <c r="AQ20" s="62"/>
+      <c r="AR20" s="62"/>
+      <c r="AS20" s="62"/>
     </row>
     <row r="21" spans="1:45" s="8" customFormat="1" ht="97" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="53"/>
       <c r="B21" s="28"/>
       <c r="C21" s="44"/>
-      <c r="D21" s="60"/>
+      <c r="D21" s="75"/>
       <c r="E21" s="28" t="s">
         <v>32</v>
       </c>
       <c r="F21" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="K21" s="89"/>
-      <c r="L21" s="89"/>
-      <c r="M21" s="89"/>
-      <c r="N21" s="89"/>
-      <c r="O21" s="89"/>
-      <c r="P21" s="89"/>
-      <c r="Q21" s="89"/>
-      <c r="R21" s="89"/>
-      <c r="S21" s="89"/>
-      <c r="T21" s="89"/>
-      <c r="U21" s="89"/>
-      <c r="V21" s="89"/>
-      <c r="W21" s="89"/>
-      <c r="X21" s="89"/>
-      <c r="Y21" s="89"/>
-      <c r="Z21" s="89"/>
-      <c r="AA21" s="89"/>
-      <c r="AB21" s="89"/>
-      <c r="AC21" s="89"/>
-      <c r="AD21" s="89"/>
-      <c r="AE21" s="89"/>
-      <c r="AF21" s="89"/>
-      <c r="AG21" s="89"/>
-      <c r="AH21" s="89"/>
-      <c r="AI21" s="89"/>
-      <c r="AJ21" s="89"/>
-      <c r="AK21" s="89"/>
-      <c r="AL21" s="89"/>
-      <c r="AM21" s="89"/>
-      <c r="AN21" s="89"/>
-      <c r="AO21" s="89"/>
-      <c r="AP21" s="89"/>
-      <c r="AQ21" s="89"/>
-      <c r="AR21" s="89"/>
-      <c r="AS21" s="89"/>
+      <c r="K21" s="62"/>
+      <c r="L21" s="62"/>
+      <c r="M21" s="62"/>
+      <c r="N21" s="62"/>
+      <c r="O21" s="62"/>
+      <c r="P21" s="62"/>
+      <c r="Q21" s="62"/>
+      <c r="R21" s="62"/>
+      <c r="S21" s="62"/>
+      <c r="T21" s="62"/>
+      <c r="U21" s="62"/>
+      <c r="V21" s="62"/>
+      <c r="W21" s="62"/>
+      <c r="X21" s="62"/>
+      <c r="Y21" s="62"/>
+      <c r="Z21" s="62"/>
+      <c r="AA21" s="62"/>
+      <c r="AB21" s="62"/>
+      <c r="AC21" s="62"/>
+      <c r="AD21" s="62"/>
+      <c r="AE21" s="62"/>
+      <c r="AF21" s="62"/>
+      <c r="AG21" s="62"/>
+      <c r="AH21" s="62"/>
+      <c r="AI21" s="62"/>
+      <c r="AJ21" s="62"/>
+      <c r="AK21" s="62"/>
+      <c r="AL21" s="62"/>
+      <c r="AM21" s="62"/>
+      <c r="AN21" s="62"/>
+      <c r="AO21" s="62"/>
+      <c r="AP21" s="62"/>
+      <c r="AQ21" s="62"/>
+      <c r="AR21" s="62"/>
+      <c r="AS21" s="62"/>
     </row>
     <row r="22" spans="1:45" s="8" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="53"/>
       <c r="B22" s="28"/>
       <c r="C22" s="44"/>
-      <c r="D22" s="65" t="s">
+      <c r="D22" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="E22" s="65"/>
-      <c r="F22" s="66"/>
-      <c r="K22" s="89"/>
-      <c r="L22" s="89"/>
-      <c r="M22" s="89"/>
-      <c r="N22" s="89"/>
-      <c r="O22" s="89"/>
-      <c r="P22" s="89"/>
-      <c r="Q22" s="89"/>
-      <c r="R22" s="89"/>
-      <c r="S22" s="89"/>
-      <c r="T22" s="89"/>
-      <c r="U22" s="89"/>
-      <c r="V22" s="89"/>
-      <c r="W22" s="89"/>
-      <c r="X22" s="89"/>
-      <c r="Y22" s="89"/>
-      <c r="Z22" s="89"/>
-      <c r="AA22" s="89"/>
-      <c r="AB22" s="89"/>
-      <c r="AC22" s="89"/>
-      <c r="AD22" s="89"/>
-      <c r="AE22" s="89"/>
-      <c r="AF22" s="89"/>
-      <c r="AG22" s="89"/>
-      <c r="AH22" s="89"/>
-      <c r="AI22" s="89"/>
-      <c r="AJ22" s="89"/>
-      <c r="AK22" s="89"/>
-      <c r="AL22" s="89"/>
-      <c r="AM22" s="89"/>
-      <c r="AN22" s="89"/>
-      <c r="AO22" s="89"/>
-      <c r="AP22" s="89"/>
-      <c r="AQ22" s="89"/>
-      <c r="AR22" s="89"/>
-      <c r="AS22" s="89"/>
+      <c r="E22" s="72"/>
+      <c r="F22" s="73"/>
+      <c r="K22" s="62"/>
+      <c r="L22" s="62"/>
+      <c r="M22" s="62"/>
+      <c r="N22" s="62"/>
+      <c r="O22" s="62"/>
+      <c r="P22" s="62"/>
+      <c r="Q22" s="62"/>
+      <c r="R22" s="62"/>
+      <c r="S22" s="62"/>
+      <c r="T22" s="62"/>
+      <c r="U22" s="62"/>
+      <c r="V22" s="62"/>
+      <c r="W22" s="62"/>
+      <c r="X22" s="62"/>
+      <c r="Y22" s="62"/>
+      <c r="Z22" s="62"/>
+      <c r="AA22" s="62"/>
+      <c r="AB22" s="62"/>
+      <c r="AC22" s="62"/>
+      <c r="AD22" s="62"/>
+      <c r="AE22" s="62"/>
+      <c r="AF22" s="62"/>
+      <c r="AG22" s="62"/>
+      <c r="AH22" s="62"/>
+      <c r="AI22" s="62"/>
+      <c r="AJ22" s="62"/>
+      <c r="AK22" s="62"/>
+      <c r="AL22" s="62"/>
+      <c r="AM22" s="62"/>
+      <c r="AN22" s="62"/>
+      <c r="AO22" s="62"/>
+      <c r="AP22" s="62"/>
+      <c r="AQ22" s="62"/>
+      <c r="AR22" s="62"/>
+      <c r="AS22" s="62"/>
     </row>
     <row r="23" spans="1:45" s="8" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="53"/>
       <c r="B23" s="28"/>
       <c r="C23" s="44"/>
-      <c r="D23" s="67" t="s">
+      <c r="D23" s="74" t="s">
         <v>23</v>
       </c>
-      <c r="E23" s="61" t="s">
+      <c r="E23" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="F23" s="62"/>
-      <c r="K23" s="89"/>
-      <c r="L23" s="89"/>
-      <c r="M23" s="89"/>
-      <c r="N23" s="89"/>
-      <c r="O23" s="89"/>
-      <c r="P23" s="89"/>
-      <c r="Q23" s="89"/>
-      <c r="R23" s="89"/>
-      <c r="S23" s="89"/>
-      <c r="T23" s="89"/>
-      <c r="U23" s="89"/>
-      <c r="V23" s="89"/>
-      <c r="W23" s="89"/>
-      <c r="X23" s="89"/>
-      <c r="Y23" s="89"/>
-      <c r="Z23" s="89"/>
-      <c r="AA23" s="89"/>
-      <c r="AB23" s="89"/>
-      <c r="AC23" s="89"/>
-      <c r="AD23" s="89"/>
-      <c r="AE23" s="89"/>
-      <c r="AF23" s="89"/>
-      <c r="AG23" s="89"/>
-      <c r="AH23" s="89"/>
-      <c r="AI23" s="89"/>
-      <c r="AJ23" s="89"/>
-      <c r="AK23" s="89"/>
-      <c r="AL23" s="89"/>
-      <c r="AM23" s="89"/>
-      <c r="AN23" s="89"/>
-      <c r="AO23" s="89"/>
-      <c r="AP23" s="89"/>
-      <c r="AQ23" s="89"/>
-      <c r="AR23" s="89"/>
-      <c r="AS23" s="89"/>
+      <c r="F23" s="69"/>
+      <c r="K23" s="62"/>
+      <c r="L23" s="62"/>
+      <c r="M23" s="62"/>
+      <c r="N23" s="62"/>
+      <c r="O23" s="62"/>
+      <c r="P23" s="62"/>
+      <c r="Q23" s="62"/>
+      <c r="R23" s="62"/>
+      <c r="S23" s="62"/>
+      <c r="T23" s="62"/>
+      <c r="U23" s="62"/>
+      <c r="V23" s="62"/>
+      <c r="W23" s="62"/>
+      <c r="X23" s="62"/>
+      <c r="Y23" s="62"/>
+      <c r="Z23" s="62"/>
+      <c r="AA23" s="62"/>
+      <c r="AB23" s="62"/>
+      <c r="AC23" s="62"/>
+      <c r="AD23" s="62"/>
+      <c r="AE23" s="62"/>
+      <c r="AF23" s="62"/>
+      <c r="AG23" s="62"/>
+      <c r="AH23" s="62"/>
+      <c r="AI23" s="62"/>
+      <c r="AJ23" s="62"/>
+      <c r="AK23" s="62"/>
+      <c r="AL23" s="62"/>
+      <c r="AM23" s="62"/>
+      <c r="AN23" s="62"/>
+      <c r="AO23" s="62"/>
+      <c r="AP23" s="62"/>
+      <c r="AQ23" s="62"/>
+      <c r="AR23" s="62"/>
+      <c r="AS23" s="62"/>
     </row>
     <row r="24" spans="1:45" s="8" customFormat="1" ht="81" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="53"/>
       <c r="B24" s="28"/>
       <c r="C24" s="44"/>
-      <c r="D24" s="60"/>
+      <c r="D24" s="75"/>
       <c r="E24" s="28" t="s">
         <v>24</v>
       </c>
       <c r="F24" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="K24" s="89"/>
-      <c r="L24" s="89"/>
-      <c r="M24" s="89"/>
-      <c r="N24" s="89"/>
-      <c r="O24" s="89"/>
-      <c r="P24" s="89"/>
-      <c r="Q24" s="89"/>
-      <c r="R24" s="89"/>
-      <c r="S24" s="89"/>
-      <c r="T24" s="89"/>
-      <c r="U24" s="89"/>
-      <c r="V24" s="89"/>
-      <c r="W24" s="89"/>
-      <c r="X24" s="89"/>
-      <c r="Y24" s="89"/>
-      <c r="Z24" s="89"/>
-      <c r="AA24" s="89"/>
-      <c r="AB24" s="89"/>
-      <c r="AC24" s="89"/>
-      <c r="AD24" s="89"/>
-      <c r="AE24" s="89"/>
-      <c r="AF24" s="89"/>
-      <c r="AG24" s="89"/>
-      <c r="AH24" s="89"/>
-      <c r="AI24" s="89"/>
-      <c r="AJ24" s="89"/>
-      <c r="AK24" s="89"/>
-      <c r="AL24" s="89"/>
-      <c r="AM24" s="89"/>
-      <c r="AN24" s="89"/>
-      <c r="AO24" s="89"/>
-      <c r="AP24" s="89"/>
-      <c r="AQ24" s="89"/>
-      <c r="AR24" s="89"/>
-      <c r="AS24" s="89"/>
+      <c r="K24" s="62"/>
+      <c r="L24" s="62"/>
+      <c r="M24" s="62"/>
+      <c r="N24" s="62"/>
+      <c r="O24" s="62"/>
+      <c r="P24" s="62"/>
+      <c r="Q24" s="62"/>
+      <c r="R24" s="62"/>
+      <c r="S24" s="62"/>
+      <c r="T24" s="62"/>
+      <c r="U24" s="62"/>
+      <c r="V24" s="62"/>
+      <c r="W24" s="62"/>
+      <c r="X24" s="62"/>
+      <c r="Y24" s="62"/>
+      <c r="Z24" s="62"/>
+      <c r="AA24" s="62"/>
+      <c r="AB24" s="62"/>
+      <c r="AC24" s="62"/>
+      <c r="AD24" s="62"/>
+      <c r="AE24" s="62"/>
+      <c r="AF24" s="62"/>
+      <c r="AG24" s="62"/>
+      <c r="AH24" s="62"/>
+      <c r="AI24" s="62"/>
+      <c r="AJ24" s="62"/>
+      <c r="AK24" s="62"/>
+      <c r="AL24" s="62"/>
+      <c r="AM24" s="62"/>
+      <c r="AN24" s="62"/>
+      <c r="AO24" s="62"/>
+      <c r="AP24" s="62"/>
+      <c r="AQ24" s="62"/>
+      <c r="AR24" s="62"/>
+      <c r="AS24" s="62"/>
     </row>
     <row r="25" spans="1:45" s="8" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="53"/>
       <c r="B25" s="28"/>
       <c r="C25" s="44"/>
-      <c r="D25" s="60"/>
-      <c r="E25" s="61" t="s">
+      <c r="D25" s="75"/>
+      <c r="E25" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="F25" s="62"/>
-      <c r="K25" s="89"/>
-      <c r="L25" s="89"/>
-      <c r="M25" s="89"/>
-      <c r="N25" s="89"/>
-      <c r="O25" s="89"/>
-      <c r="P25" s="89"/>
-      <c r="Q25" s="89"/>
-      <c r="R25" s="89"/>
-      <c r="S25" s="89"/>
-      <c r="T25" s="89"/>
-      <c r="U25" s="89"/>
-      <c r="V25" s="89"/>
-      <c r="W25" s="89"/>
-      <c r="X25" s="89"/>
-      <c r="Y25" s="89"/>
-      <c r="Z25" s="89"/>
-      <c r="AA25" s="89"/>
-      <c r="AB25" s="89"/>
-      <c r="AC25" s="89"/>
-      <c r="AD25" s="89"/>
-      <c r="AE25" s="89"/>
-      <c r="AF25" s="89"/>
-      <c r="AG25" s="89"/>
-      <c r="AH25" s="89"/>
-      <c r="AI25" s="89"/>
-      <c r="AJ25" s="89"/>
-      <c r="AK25" s="89"/>
-      <c r="AL25" s="89"/>
-      <c r="AM25" s="89"/>
-      <c r="AN25" s="89"/>
-      <c r="AO25" s="89"/>
-      <c r="AP25" s="89"/>
-      <c r="AQ25" s="89"/>
-      <c r="AR25" s="89"/>
-      <c r="AS25" s="89"/>
+      <c r="F25" s="69"/>
+      <c r="K25" s="62"/>
+      <c r="L25" s="62"/>
+      <c r="M25" s="62"/>
+      <c r="N25" s="62"/>
+      <c r="O25" s="62"/>
+      <c r="P25" s="62"/>
+      <c r="Q25" s="62"/>
+      <c r="R25" s="62"/>
+      <c r="S25" s="62"/>
+      <c r="T25" s="62"/>
+      <c r="U25" s="62"/>
+      <c r="V25" s="62"/>
+      <c r="W25" s="62"/>
+      <c r="X25" s="62"/>
+      <c r="Y25" s="62"/>
+      <c r="Z25" s="62"/>
+      <c r="AA25" s="62"/>
+      <c r="AB25" s="62"/>
+      <c r="AC25" s="62"/>
+      <c r="AD25" s="62"/>
+      <c r="AE25" s="62"/>
+      <c r="AF25" s="62"/>
+      <c r="AG25" s="62"/>
+      <c r="AH25" s="62"/>
+      <c r="AI25" s="62"/>
+      <c r="AJ25" s="62"/>
+      <c r="AK25" s="62"/>
+      <c r="AL25" s="62"/>
+      <c r="AM25" s="62"/>
+      <c r="AN25" s="62"/>
+      <c r="AO25" s="62"/>
+      <c r="AP25" s="62"/>
+      <c r="AQ25" s="62"/>
+      <c r="AR25" s="62"/>
+      <c r="AS25" s="62"/>
     </row>
     <row r="26" spans="1:45" s="8" customFormat="1" ht="61" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="53"/>
       <c r="B26" s="28"/>
       <c r="C26" s="44"/>
-      <c r="D26" s="60"/>
+      <c r="D26" s="75"/>
       <c r="E26" s="28" t="s">
         <v>26</v>
       </c>
       <c r="F26" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="K26" s="89"/>
-      <c r="L26" s="89"/>
-      <c r="M26" s="89"/>
-      <c r="N26" s="89"/>
-      <c r="O26" s="89"/>
-      <c r="P26" s="89"/>
-      <c r="Q26" s="89"/>
-      <c r="R26" s="89"/>
-      <c r="S26" s="89"/>
-      <c r="T26" s="89"/>
-      <c r="U26" s="89"/>
-      <c r="V26" s="89"/>
-      <c r="W26" s="89"/>
-      <c r="X26" s="89"/>
-      <c r="Y26" s="89"/>
-      <c r="Z26" s="89"/>
-      <c r="AA26" s="89"/>
-      <c r="AB26" s="89"/>
-      <c r="AC26" s="89"/>
-      <c r="AD26" s="89"/>
-      <c r="AE26" s="89"/>
-      <c r="AF26" s="89"/>
-      <c r="AG26" s="89"/>
-      <c r="AH26" s="89"/>
-      <c r="AI26" s="89"/>
-      <c r="AJ26" s="89"/>
-      <c r="AK26" s="89"/>
-      <c r="AL26" s="89"/>
-      <c r="AM26" s="89"/>
-      <c r="AN26" s="89"/>
-      <c r="AO26" s="89"/>
-      <c r="AP26" s="89"/>
-      <c r="AQ26" s="89"/>
-      <c r="AR26" s="89"/>
-      <c r="AS26" s="89"/>
+      <c r="K26" s="62"/>
+      <c r="L26" s="62"/>
+      <c r="M26" s="62"/>
+      <c r="N26" s="62"/>
+      <c r="O26" s="62"/>
+      <c r="P26" s="62"/>
+      <c r="Q26" s="62"/>
+      <c r="R26" s="62"/>
+      <c r="S26" s="62"/>
+      <c r="T26" s="62"/>
+      <c r="U26" s="62"/>
+      <c r="V26" s="62"/>
+      <c r="W26" s="62"/>
+      <c r="X26" s="62"/>
+      <c r="Y26" s="62"/>
+      <c r="Z26" s="62"/>
+      <c r="AA26" s="62"/>
+      <c r="AB26" s="62"/>
+      <c r="AC26" s="62"/>
+      <c r="AD26" s="62"/>
+      <c r="AE26" s="62"/>
+      <c r="AF26" s="62"/>
+      <c r="AG26" s="62"/>
+      <c r="AH26" s="62"/>
+      <c r="AI26" s="62"/>
+      <c r="AJ26" s="62"/>
+      <c r="AK26" s="62"/>
+      <c r="AL26" s="62"/>
+      <c r="AM26" s="62"/>
+      <c r="AN26" s="62"/>
+      <c r="AO26" s="62"/>
+      <c r="AP26" s="62"/>
+      <c r="AQ26" s="62"/>
+      <c r="AR26" s="62"/>
+      <c r="AS26" s="62"/>
     </row>
     <row r="27" spans="1:45" s="8" customFormat="1" ht="23" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="53"/>
       <c r="B27" s="28"/>
       <c r="C27" s="44"/>
-      <c r="D27" s="65" t="s">
+      <c r="D27" s="72" t="s">
         <v>12</v>
       </c>
-      <c r="E27" s="65"/>
-      <c r="F27" s="66"/>
-      <c r="K27" s="89"/>
-      <c r="L27" s="89"/>
-      <c r="M27" s="89"/>
-      <c r="N27" s="89"/>
-      <c r="O27" s="89"/>
-      <c r="P27" s="89"/>
-      <c r="Q27" s="89"/>
-      <c r="R27" s="89"/>
-      <c r="S27" s="89"/>
-      <c r="T27" s="89"/>
-      <c r="U27" s="89"/>
-      <c r="V27" s="89"/>
-      <c r="W27" s="89"/>
-      <c r="X27" s="89"/>
-      <c r="Y27" s="89"/>
-      <c r="Z27" s="89"/>
-      <c r="AA27" s="89"/>
-      <c r="AB27" s="89"/>
-      <c r="AC27" s="89"/>
-      <c r="AD27" s="89"/>
-      <c r="AE27" s="89"/>
-      <c r="AF27" s="89"/>
-      <c r="AG27" s="89"/>
-      <c r="AH27" s="89"/>
-      <c r="AI27" s="89"/>
-      <c r="AJ27" s="89"/>
-      <c r="AK27" s="89"/>
-      <c r="AL27" s="89"/>
-      <c r="AM27" s="89"/>
-      <c r="AN27" s="89"/>
-      <c r="AO27" s="89"/>
-      <c r="AP27" s="89"/>
-      <c r="AQ27" s="89"/>
-      <c r="AR27" s="89"/>
-      <c r="AS27" s="89"/>
+      <c r="E27" s="72"/>
+      <c r="F27" s="73"/>
+      <c r="K27" s="62"/>
+      <c r="L27" s="62"/>
+      <c r="M27" s="62"/>
+      <c r="N27" s="62"/>
+      <c r="O27" s="62"/>
+      <c r="P27" s="62"/>
+      <c r="Q27" s="62"/>
+      <c r="R27" s="62"/>
+      <c r="S27" s="62"/>
+      <c r="T27" s="62"/>
+      <c r="U27" s="62"/>
+      <c r="V27" s="62"/>
+      <c r="W27" s="62"/>
+      <c r="X27" s="62"/>
+      <c r="Y27" s="62"/>
+      <c r="Z27" s="62"/>
+      <c r="AA27" s="62"/>
+      <c r="AB27" s="62"/>
+      <c r="AC27" s="62"/>
+      <c r="AD27" s="62"/>
+      <c r="AE27" s="62"/>
+      <c r="AF27" s="62"/>
+      <c r="AG27" s="62"/>
+      <c r="AH27" s="62"/>
+      <c r="AI27" s="62"/>
+      <c r="AJ27" s="62"/>
+      <c r="AK27" s="62"/>
+      <c r="AL27" s="62"/>
+      <c r="AM27" s="62"/>
+      <c r="AN27" s="62"/>
+      <c r="AO27" s="62"/>
+      <c r="AP27" s="62"/>
+      <c r="AQ27" s="62"/>
+      <c r="AR27" s="62"/>
+      <c r="AS27" s="62"/>
     </row>
     <row r="28" spans="1:45" s="8" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="53"/>
       <c r="B28" s="28"/>
       <c r="C28" s="44"/>
-      <c r="D28" s="68" t="s">
+      <c r="D28" s="76" t="s">
         <v>42</v>
       </c>
-      <c r="E28" s="61" t="s">
+      <c r="E28" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="F28" s="62"/>
-      <c r="K28" s="89"/>
-      <c r="L28" s="89"/>
-      <c r="M28" s="89"/>
-      <c r="N28" s="89"/>
-      <c r="O28" s="89"/>
-      <c r="P28" s="89"/>
-      <c r="Q28" s="89"/>
-      <c r="R28" s="89"/>
-      <c r="S28" s="89"/>
-      <c r="T28" s="89"/>
-      <c r="U28" s="89"/>
-      <c r="V28" s="89"/>
-      <c r="W28" s="89"/>
-      <c r="X28" s="89"/>
-      <c r="Y28" s="89"/>
-      <c r="Z28" s="89"/>
-      <c r="AA28" s="89"/>
-      <c r="AB28" s="89"/>
-      <c r="AC28" s="89"/>
-      <c r="AD28" s="89"/>
-      <c r="AE28" s="89"/>
-      <c r="AF28" s="89"/>
-      <c r="AG28" s="89"/>
-      <c r="AH28" s="89"/>
-      <c r="AI28" s="89"/>
-      <c r="AJ28" s="89"/>
-      <c r="AK28" s="89"/>
-      <c r="AL28" s="89"/>
-      <c r="AM28" s="89"/>
-      <c r="AN28" s="89"/>
-      <c r="AO28" s="89"/>
-      <c r="AP28" s="89"/>
-      <c r="AQ28" s="89"/>
-      <c r="AR28" s="89"/>
-      <c r="AS28" s="89"/>
+      <c r="F28" s="69"/>
+      <c r="K28" s="62"/>
+      <c r="L28" s="62"/>
+      <c r="M28" s="62"/>
+      <c r="N28" s="62"/>
+      <c r="O28" s="62"/>
+      <c r="P28" s="62"/>
+      <c r="Q28" s="62"/>
+      <c r="R28" s="62"/>
+      <c r="S28" s="62"/>
+      <c r="T28" s="62"/>
+      <c r="U28" s="62"/>
+      <c r="V28" s="62"/>
+      <c r="W28" s="62"/>
+      <c r="X28" s="62"/>
+      <c r="Y28" s="62"/>
+      <c r="Z28" s="62"/>
+      <c r="AA28" s="62"/>
+      <c r="AB28" s="62"/>
+      <c r="AC28" s="62"/>
+      <c r="AD28" s="62"/>
+      <c r="AE28" s="62"/>
+      <c r="AF28" s="62"/>
+      <c r="AG28" s="62"/>
+      <c r="AH28" s="62"/>
+      <c r="AI28" s="62"/>
+      <c r="AJ28" s="62"/>
+      <c r="AK28" s="62"/>
+      <c r="AL28" s="62"/>
+      <c r="AM28" s="62"/>
+      <c r="AN28" s="62"/>
+      <c r="AO28" s="62"/>
+      <c r="AP28" s="62"/>
+      <c r="AQ28" s="62"/>
+      <c r="AR28" s="62"/>
+      <c r="AS28" s="62"/>
     </row>
     <row r="29" spans="1:45" s="8" customFormat="1" ht="130" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="53"/>
       <c r="B29" s="28"/>
       <c r="C29" s="44"/>
-      <c r="D29" s="69"/>
+      <c r="D29" s="77"/>
       <c r="E29" s="28" t="s">
         <v>43</v>
       </c>
       <c r="F29" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="K29" s="89"/>
-      <c r="L29" s="89"/>
-      <c r="M29" s="89"/>
-      <c r="N29" s="89"/>
-      <c r="O29" s="89"/>
-      <c r="P29" s="89"/>
-      <c r="Q29" s="89"/>
-      <c r="R29" s="89"/>
-      <c r="S29" s="89"/>
-      <c r="T29" s="89"/>
-      <c r="U29" s="89"/>
-      <c r="V29" s="89"/>
-      <c r="W29" s="89"/>
-      <c r="X29" s="89"/>
-      <c r="Y29" s="89"/>
-      <c r="Z29" s="89"/>
-      <c r="AA29" s="89"/>
-      <c r="AB29" s="89"/>
-      <c r="AC29" s="89"/>
-      <c r="AD29" s="89"/>
-      <c r="AE29" s="89"/>
-      <c r="AF29" s="89"/>
-      <c r="AG29" s="89"/>
-      <c r="AH29" s="89"/>
-      <c r="AI29" s="89"/>
-      <c r="AJ29" s="89"/>
-      <c r="AK29" s="89"/>
-      <c r="AL29" s="89"/>
-      <c r="AM29" s="89"/>
-      <c r="AN29" s="89"/>
-      <c r="AO29" s="89"/>
-      <c r="AP29" s="89"/>
-      <c r="AQ29" s="89"/>
-      <c r="AR29" s="89"/>
-      <c r="AS29" s="89"/>
+      <c r="K29" s="62"/>
+      <c r="L29" s="62"/>
+      <c r="M29" s="62"/>
+      <c r="N29" s="62"/>
+      <c r="O29" s="62"/>
+      <c r="P29" s="62"/>
+      <c r="Q29" s="62"/>
+      <c r="R29" s="62"/>
+      <c r="S29" s="62"/>
+      <c r="T29" s="62"/>
+      <c r="U29" s="62"/>
+      <c r="V29" s="62"/>
+      <c r="W29" s="62"/>
+      <c r="X29" s="62"/>
+      <c r="Y29" s="62"/>
+      <c r="Z29" s="62"/>
+      <c r="AA29" s="62"/>
+      <c r="AB29" s="62"/>
+      <c r="AC29" s="62"/>
+      <c r="AD29" s="62"/>
+      <c r="AE29" s="62"/>
+      <c r="AF29" s="62"/>
+      <c r="AG29" s="62"/>
+      <c r="AH29" s="62"/>
+      <c r="AI29" s="62"/>
+      <c r="AJ29" s="62"/>
+      <c r="AK29" s="62"/>
+      <c r="AL29" s="62"/>
+      <c r="AM29" s="62"/>
+      <c r="AN29" s="62"/>
+      <c r="AO29" s="62"/>
+      <c r="AP29" s="62"/>
+      <c r="AQ29" s="62"/>
+      <c r="AR29" s="62"/>
+      <c r="AS29" s="62"/>
     </row>
     <row r="30" spans="1:45" s="8" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="53"/>
       <c r="B30" s="28"/>
       <c r="C30" s="44"/>
-      <c r="D30" s="69"/>
-      <c r="E30" s="61" t="s">
+      <c r="D30" s="77"/>
+      <c r="E30" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="F30" s="62"/>
-      <c r="K30" s="89"/>
-      <c r="L30" s="89"/>
-      <c r="M30" s="89"/>
-      <c r="N30" s="89"/>
-      <c r="O30" s="89"/>
-      <c r="P30" s="89"/>
-      <c r="Q30" s="89"/>
-      <c r="R30" s="89"/>
-      <c r="S30" s="89"/>
-      <c r="T30" s="89"/>
-      <c r="U30" s="89"/>
-      <c r="V30" s="89"/>
-      <c r="W30" s="89"/>
-      <c r="X30" s="89"/>
-      <c r="Y30" s="89"/>
-      <c r="Z30" s="89"/>
-      <c r="AA30" s="89"/>
-      <c r="AB30" s="89"/>
-      <c r="AC30" s="89"/>
-      <c r="AD30" s="89"/>
-      <c r="AE30" s="89"/>
-      <c r="AF30" s="89"/>
-      <c r="AG30" s="89"/>
-      <c r="AH30" s="89"/>
-      <c r="AI30" s="89"/>
-      <c r="AJ30" s="89"/>
-      <c r="AK30" s="89"/>
-      <c r="AL30" s="89"/>
-      <c r="AM30" s="89"/>
-      <c r="AN30" s="89"/>
-      <c r="AO30" s="89"/>
-      <c r="AP30" s="89"/>
-      <c r="AQ30" s="89"/>
-      <c r="AR30" s="89"/>
-      <c r="AS30" s="89"/>
+      <c r="F30" s="69"/>
+      <c r="K30" s="62"/>
+      <c r="L30" s="62"/>
+      <c r="M30" s="62"/>
+      <c r="N30" s="62"/>
+      <c r="O30" s="62"/>
+      <c r="P30" s="62"/>
+      <c r="Q30" s="62"/>
+      <c r="R30" s="62"/>
+      <c r="S30" s="62"/>
+      <c r="T30" s="62"/>
+      <c r="U30" s="62"/>
+      <c r="V30" s="62"/>
+      <c r="W30" s="62"/>
+      <c r="X30" s="62"/>
+      <c r="Y30" s="62"/>
+      <c r="Z30" s="62"/>
+      <c r="AA30" s="62"/>
+      <c r="AB30" s="62"/>
+      <c r="AC30" s="62"/>
+      <c r="AD30" s="62"/>
+      <c r="AE30" s="62"/>
+      <c r="AF30" s="62"/>
+      <c r="AG30" s="62"/>
+      <c r="AH30" s="62"/>
+      <c r="AI30" s="62"/>
+      <c r="AJ30" s="62"/>
+      <c r="AK30" s="62"/>
+      <c r="AL30" s="62"/>
+      <c r="AM30" s="62"/>
+      <c r="AN30" s="62"/>
+      <c r="AO30" s="62"/>
+      <c r="AP30" s="62"/>
+      <c r="AQ30" s="62"/>
+      <c r="AR30" s="62"/>
+      <c r="AS30" s="62"/>
     </row>
     <row r="31" spans="1:45" s="8" customFormat="1" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="53"/>
       <c r="B31" s="28"/>
       <c r="C31" s="44"/>
-      <c r="D31" s="70"/>
+      <c r="D31" s="78"/>
       <c r="E31" s="34"/>
       <c r="F31" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="K31" s="89"/>
-      <c r="L31" s="89"/>
-      <c r="M31" s="89"/>
-      <c r="N31" s="89"/>
-      <c r="O31" s="89"/>
-      <c r="P31" s="89"/>
-      <c r="Q31" s="89"/>
-      <c r="R31" s="89"/>
-      <c r="S31" s="89"/>
-      <c r="T31" s="89"/>
-      <c r="U31" s="89"/>
-      <c r="V31" s="89"/>
-      <c r="W31" s="89"/>
-      <c r="X31" s="89"/>
-      <c r="Y31" s="89"/>
-      <c r="Z31" s="89"/>
-      <c r="AA31" s="89"/>
-      <c r="AB31" s="89"/>
-      <c r="AC31" s="89"/>
-      <c r="AD31" s="89"/>
-      <c r="AE31" s="89"/>
-      <c r="AF31" s="89"/>
-      <c r="AG31" s="89"/>
-      <c r="AH31" s="89"/>
-      <c r="AI31" s="89"/>
-      <c r="AJ31" s="89"/>
-      <c r="AK31" s="89"/>
-      <c r="AL31" s="89"/>
-      <c r="AM31" s="89"/>
-      <c r="AN31" s="89"/>
-      <c r="AO31" s="89"/>
-      <c r="AP31" s="89"/>
-      <c r="AQ31" s="89"/>
-      <c r="AR31" s="89"/>
-      <c r="AS31" s="89"/>
+      <c r="K31" s="62"/>
+      <c r="L31" s="62"/>
+      <c r="M31" s="62"/>
+      <c r="N31" s="62"/>
+      <c r="O31" s="62"/>
+      <c r="P31" s="62"/>
+      <c r="Q31" s="62"/>
+      <c r="R31" s="62"/>
+      <c r="S31" s="62"/>
+      <c r="T31" s="62"/>
+      <c r="U31" s="62"/>
+      <c r="V31" s="62"/>
+      <c r="W31" s="62"/>
+      <c r="X31" s="62"/>
+      <c r="Y31" s="62"/>
+      <c r="Z31" s="62"/>
+      <c r="AA31" s="62"/>
+      <c r="AB31" s="62"/>
+      <c r="AC31" s="62"/>
+      <c r="AD31" s="62"/>
+      <c r="AE31" s="62"/>
+      <c r="AF31" s="62"/>
+      <c r="AG31" s="62"/>
+      <c r="AH31" s="62"/>
+      <c r="AI31" s="62"/>
+      <c r="AJ31" s="62"/>
+      <c r="AK31" s="62"/>
+      <c r="AL31" s="62"/>
+      <c r="AM31" s="62"/>
+      <c r="AN31" s="62"/>
+      <c r="AO31" s="62"/>
+      <c r="AP31" s="62"/>
+      <c r="AQ31" s="62"/>
+      <c r="AR31" s="62"/>
+      <c r="AS31" s="62"/>
     </row>
     <row r="32" spans="1:45" ht="66" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="53"/>
@@ -2785,44 +2785,44 @@
       <c r="C32" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="D32" s="73"/>
-      <c r="E32" s="74"/>
-      <c r="F32" s="75"/>
-      <c r="K32" s="86"/>
-      <c r="L32" s="86"/>
-      <c r="M32" s="86"/>
-      <c r="N32" s="86"/>
-      <c r="O32" s="86"/>
-      <c r="P32" s="86"/>
-      <c r="Q32" s="86"/>
-      <c r="R32" s="86"/>
-      <c r="S32" s="86"/>
-      <c r="T32" s="86"/>
-      <c r="U32" s="86"/>
-      <c r="V32" s="86"/>
-      <c r="W32" s="86"/>
-      <c r="X32" s="86"/>
-      <c r="Y32" s="86"/>
-      <c r="Z32" s="86"/>
-      <c r="AA32" s="86"/>
-      <c r="AB32" s="86"/>
-      <c r="AC32" s="86"/>
-      <c r="AD32" s="86"/>
-      <c r="AE32" s="86"/>
-      <c r="AF32" s="86"/>
-      <c r="AG32" s="86"/>
-      <c r="AH32" s="86"/>
-      <c r="AI32" s="86"/>
-      <c r="AJ32" s="86"/>
-      <c r="AK32" s="86"/>
-      <c r="AL32" s="86"/>
-      <c r="AM32" s="86"/>
-      <c r="AN32" s="86"/>
-      <c r="AO32" s="86"/>
-      <c r="AP32" s="86"/>
-      <c r="AQ32" s="86"/>
-      <c r="AR32" s="86"/>
-      <c r="AS32" s="86"/>
+      <c r="D32" s="63"/>
+      <c r="E32" s="64"/>
+      <c r="F32" s="65"/>
+      <c r="K32" s="59"/>
+      <c r="L32" s="59"/>
+      <c r="M32" s="59"/>
+      <c r="N32" s="59"/>
+      <c r="O32" s="59"/>
+      <c r="P32" s="59"/>
+      <c r="Q32" s="59"/>
+      <c r="R32" s="59"/>
+      <c r="S32" s="59"/>
+      <c r="T32" s="59"/>
+      <c r="U32" s="59"/>
+      <c r="V32" s="59"/>
+      <c r="W32" s="59"/>
+      <c r="X32" s="59"/>
+      <c r="Y32" s="59"/>
+      <c r="Z32" s="59"/>
+      <c r="AA32" s="59"/>
+      <c r="AB32" s="59"/>
+      <c r="AC32" s="59"/>
+      <c r="AD32" s="59"/>
+      <c r="AE32" s="59"/>
+      <c r="AF32" s="59"/>
+      <c r="AG32" s="59"/>
+      <c r="AH32" s="59"/>
+      <c r="AI32" s="59"/>
+      <c r="AJ32" s="59"/>
+      <c r="AK32" s="59"/>
+      <c r="AL32" s="59"/>
+      <c r="AM32" s="59"/>
+      <c r="AN32" s="59"/>
+      <c r="AO32" s="59"/>
+      <c r="AP32" s="59"/>
+      <c r="AQ32" s="59"/>
+      <c r="AR32" s="59"/>
+      <c r="AS32" s="59"/>
     </row>
     <row r="33" spans="1:45" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="53"/>
@@ -2833,41 +2833,41 @@
       </c>
       <c r="E33" s="17"/>
       <c r="F33" s="17"/>
-      <c r="K33" s="86"/>
-      <c r="L33" s="86"/>
-      <c r="M33" s="86"/>
-      <c r="N33" s="86"/>
-      <c r="O33" s="86"/>
-      <c r="P33" s="86"/>
-      <c r="Q33" s="86"/>
-      <c r="R33" s="86"/>
-      <c r="S33" s="86"/>
-      <c r="T33" s="86"/>
-      <c r="U33" s="86"/>
-      <c r="V33" s="86"/>
-      <c r="W33" s="86"/>
-      <c r="X33" s="86"/>
-      <c r="Y33" s="86"/>
-      <c r="Z33" s="86"/>
-      <c r="AA33" s="86"/>
-      <c r="AB33" s="86"/>
-      <c r="AC33" s="86"/>
-      <c r="AD33" s="86"/>
-      <c r="AE33" s="86"/>
-      <c r="AF33" s="86"/>
-      <c r="AG33" s="86"/>
-      <c r="AH33" s="86"/>
-      <c r="AI33" s="86"/>
-      <c r="AJ33" s="86"/>
-      <c r="AK33" s="86"/>
-      <c r="AL33" s="86"/>
-      <c r="AM33" s="86"/>
-      <c r="AN33" s="86"/>
-      <c r="AO33" s="86"/>
-      <c r="AP33" s="86"/>
-      <c r="AQ33" s="86"/>
-      <c r="AR33" s="86"/>
-      <c r="AS33" s="86"/>
+      <c r="K33" s="59"/>
+      <c r="L33" s="59"/>
+      <c r="M33" s="59"/>
+      <c r="N33" s="59"/>
+      <c r="O33" s="59"/>
+      <c r="P33" s="59"/>
+      <c r="Q33" s="59"/>
+      <c r="R33" s="59"/>
+      <c r="S33" s="59"/>
+      <c r="T33" s="59"/>
+      <c r="U33" s="59"/>
+      <c r="V33" s="59"/>
+      <c r="W33" s="59"/>
+      <c r="X33" s="59"/>
+      <c r="Y33" s="59"/>
+      <c r="Z33" s="59"/>
+      <c r="AA33" s="59"/>
+      <c r="AB33" s="59"/>
+      <c r="AC33" s="59"/>
+      <c r="AD33" s="59"/>
+      <c r="AE33" s="59"/>
+      <c r="AF33" s="59"/>
+      <c r="AG33" s="59"/>
+      <c r="AH33" s="59"/>
+      <c r="AI33" s="59"/>
+      <c r="AJ33" s="59"/>
+      <c r="AK33" s="59"/>
+      <c r="AL33" s="59"/>
+      <c r="AM33" s="59"/>
+      <c r="AN33" s="59"/>
+      <c r="AO33" s="59"/>
+      <c r="AP33" s="59"/>
+      <c r="AQ33" s="59"/>
+      <c r="AR33" s="59"/>
+      <c r="AS33" s="59"/>
     </row>
     <row r="34" spans="1:45" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="53"/>
@@ -2876,41 +2876,41 @@
       <c r="D34" s="19"/>
       <c r="E34" s="15"/>
       <c r="F34" s="15"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="86"/>
-      <c r="M34" s="86"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="86"/>
-      <c r="P34" s="86"/>
-      <c r="Q34" s="86"/>
-      <c r="R34" s="86"/>
-      <c r="S34" s="86"/>
-      <c r="T34" s="86"/>
-      <c r="U34" s="86"/>
-      <c r="V34" s="86"/>
-      <c r="W34" s="86"/>
-      <c r="X34" s="86"/>
-      <c r="Y34" s="86"/>
-      <c r="Z34" s="86"/>
-      <c r="AA34" s="86"/>
-      <c r="AB34" s="86"/>
-      <c r="AC34" s="86"/>
-      <c r="AD34" s="86"/>
-      <c r="AE34" s="86"/>
-      <c r="AF34" s="86"/>
-      <c r="AG34" s="86"/>
-      <c r="AH34" s="86"/>
-      <c r="AI34" s="86"/>
-      <c r="AJ34" s="86"/>
-      <c r="AK34" s="86"/>
-      <c r="AL34" s="86"/>
-      <c r="AM34" s="86"/>
-      <c r="AN34" s="86"/>
-      <c r="AO34" s="86"/>
-      <c r="AP34" s="86"/>
-      <c r="AQ34" s="86"/>
-      <c r="AR34" s="86"/>
-      <c r="AS34" s="86"/>
+      <c r="K34" s="59"/>
+      <c r="L34" s="59"/>
+      <c r="M34" s="59"/>
+      <c r="N34" s="59"/>
+      <c r="O34" s="59"/>
+      <c r="P34" s="59"/>
+      <c r="Q34" s="59"/>
+      <c r="R34" s="59"/>
+      <c r="S34" s="59"/>
+      <c r="T34" s="59"/>
+      <c r="U34" s="59"/>
+      <c r="V34" s="59"/>
+      <c r="W34" s="59"/>
+      <c r="X34" s="59"/>
+      <c r="Y34" s="59"/>
+      <c r="Z34" s="59"/>
+      <c r="AA34" s="59"/>
+      <c r="AB34" s="59"/>
+      <c r="AC34" s="59"/>
+      <c r="AD34" s="59"/>
+      <c r="AE34" s="59"/>
+      <c r="AF34" s="59"/>
+      <c r="AG34" s="59"/>
+      <c r="AH34" s="59"/>
+      <c r="AI34" s="59"/>
+      <c r="AJ34" s="59"/>
+      <c r="AK34" s="59"/>
+      <c r="AL34" s="59"/>
+      <c r="AM34" s="59"/>
+      <c r="AN34" s="59"/>
+      <c r="AO34" s="59"/>
+      <c r="AP34" s="59"/>
+      <c r="AQ34" s="59"/>
+      <c r="AR34" s="59"/>
+      <c r="AS34" s="59"/>
     </row>
     <row r="35" spans="1:45" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="53"/>
@@ -2921,41 +2921,41 @@
       </c>
       <c r="E35" s="17"/>
       <c r="F35" s="17"/>
-      <c r="K35" s="86"/>
-      <c r="L35" s="86"/>
-      <c r="M35" s="86"/>
-      <c r="N35" s="86"/>
-      <c r="O35" s="86"/>
-      <c r="P35" s="86"/>
-      <c r="Q35" s="86"/>
-      <c r="R35" s="86"/>
-      <c r="S35" s="86"/>
-      <c r="T35" s="86"/>
-      <c r="U35" s="86"/>
-      <c r="V35" s="86"/>
-      <c r="W35" s="86"/>
-      <c r="X35" s="86"/>
-      <c r="Y35" s="86"/>
-      <c r="Z35" s="86"/>
-      <c r="AA35" s="86"/>
-      <c r="AB35" s="86"/>
-      <c r="AC35" s="86"/>
-      <c r="AD35" s="86"/>
-      <c r="AE35" s="86"/>
-      <c r="AF35" s="86"/>
-      <c r="AG35" s="86"/>
-      <c r="AH35" s="86"/>
-      <c r="AI35" s="86"/>
-      <c r="AJ35" s="86"/>
-      <c r="AK35" s="86"/>
-      <c r="AL35" s="86"/>
-      <c r="AM35" s="86"/>
-      <c r="AN35" s="86"/>
-      <c r="AO35" s="86"/>
-      <c r="AP35" s="86"/>
-      <c r="AQ35" s="86"/>
-      <c r="AR35" s="86"/>
-      <c r="AS35" s="86"/>
+      <c r="K35" s="59"/>
+      <c r="L35" s="59"/>
+      <c r="M35" s="59"/>
+      <c r="N35" s="59"/>
+      <c r="O35" s="59"/>
+      <c r="P35" s="59"/>
+      <c r="Q35" s="59"/>
+      <c r="R35" s="59"/>
+      <c r="S35" s="59"/>
+      <c r="T35" s="59"/>
+      <c r="U35" s="59"/>
+      <c r="V35" s="59"/>
+      <c r="W35" s="59"/>
+      <c r="X35" s="59"/>
+      <c r="Y35" s="59"/>
+      <c r="Z35" s="59"/>
+      <c r="AA35" s="59"/>
+      <c r="AB35" s="59"/>
+      <c r="AC35" s="59"/>
+      <c r="AD35" s="59"/>
+      <c r="AE35" s="59"/>
+      <c r="AF35" s="59"/>
+      <c r="AG35" s="59"/>
+      <c r="AH35" s="59"/>
+      <c r="AI35" s="59"/>
+      <c r="AJ35" s="59"/>
+      <c r="AK35" s="59"/>
+      <c r="AL35" s="59"/>
+      <c r="AM35" s="59"/>
+      <c r="AN35" s="59"/>
+      <c r="AO35" s="59"/>
+      <c r="AP35" s="59"/>
+      <c r="AQ35" s="59"/>
+      <c r="AR35" s="59"/>
+      <c r="AS35" s="59"/>
     </row>
     <row r="36" spans="1:45" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="53"/>
@@ -2964,41 +2964,41 @@
       <c r="D36" s="19"/>
       <c r="E36" s="15"/>
       <c r="F36" s="15"/>
-      <c r="K36" s="86"/>
-      <c r="L36" s="86"/>
-      <c r="M36" s="86"/>
-      <c r="N36" s="86"/>
-      <c r="O36" s="86"/>
-      <c r="P36" s="86"/>
-      <c r="Q36" s="86"/>
-      <c r="R36" s="86"/>
-      <c r="S36" s="86"/>
-      <c r="T36" s="86"/>
-      <c r="U36" s="86"/>
-      <c r="V36" s="86"/>
-      <c r="W36" s="86"/>
-      <c r="X36" s="86"/>
-      <c r="Y36" s="86"/>
-      <c r="Z36" s="86"/>
-      <c r="AA36" s="86"/>
-      <c r="AB36" s="86"/>
-      <c r="AC36" s="86"/>
-      <c r="AD36" s="86"/>
-      <c r="AE36" s="86"/>
-      <c r="AF36" s="86"/>
-      <c r="AG36" s="86"/>
-      <c r="AH36" s="86"/>
-      <c r="AI36" s="86"/>
-      <c r="AJ36" s="86"/>
-      <c r="AK36" s="86"/>
-      <c r="AL36" s="86"/>
-      <c r="AM36" s="86"/>
-      <c r="AN36" s="86"/>
-      <c r="AO36" s="86"/>
-      <c r="AP36" s="86"/>
-      <c r="AQ36" s="86"/>
-      <c r="AR36" s="86"/>
-      <c r="AS36" s="86"/>
+      <c r="K36" s="59"/>
+      <c r="L36" s="59"/>
+      <c r="M36" s="59"/>
+      <c r="N36" s="59"/>
+      <c r="O36" s="59"/>
+      <c r="P36" s="59"/>
+      <c r="Q36" s="59"/>
+      <c r="R36" s="59"/>
+      <c r="S36" s="59"/>
+      <c r="T36" s="59"/>
+      <c r="U36" s="59"/>
+      <c r="V36" s="59"/>
+      <c r="W36" s="59"/>
+      <c r="X36" s="59"/>
+      <c r="Y36" s="59"/>
+      <c r="Z36" s="59"/>
+      <c r="AA36" s="59"/>
+      <c r="AB36" s="59"/>
+      <c r="AC36" s="59"/>
+      <c r="AD36" s="59"/>
+      <c r="AE36" s="59"/>
+      <c r="AF36" s="59"/>
+      <c r="AG36" s="59"/>
+      <c r="AH36" s="59"/>
+      <c r="AI36" s="59"/>
+      <c r="AJ36" s="59"/>
+      <c r="AK36" s="59"/>
+      <c r="AL36" s="59"/>
+      <c r="AM36" s="59"/>
+      <c r="AN36" s="59"/>
+      <c r="AO36" s="59"/>
+      <c r="AP36" s="59"/>
+      <c r="AQ36" s="59"/>
+      <c r="AR36" s="59"/>
+      <c r="AS36" s="59"/>
     </row>
     <row r="37" spans="1:45" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="53"/>
@@ -3009,41 +3009,41 @@
       </c>
       <c r="E37" s="17"/>
       <c r="F37" s="17"/>
-      <c r="K37" s="86"/>
-      <c r="L37" s="86"/>
-      <c r="M37" s="86"/>
-      <c r="N37" s="86"/>
-      <c r="O37" s="86"/>
-      <c r="P37" s="86"/>
-      <c r="Q37" s="86"/>
-      <c r="R37" s="86"/>
-      <c r="S37" s="86"/>
-      <c r="T37" s="86"/>
-      <c r="U37" s="86"/>
-      <c r="V37" s="86"/>
-      <c r="W37" s="86"/>
-      <c r="X37" s="86"/>
-      <c r="Y37" s="86"/>
-      <c r="Z37" s="86"/>
-      <c r="AA37" s="86"/>
-      <c r="AB37" s="86"/>
-      <c r="AC37" s="86"/>
-      <c r="AD37" s="86"/>
-      <c r="AE37" s="86"/>
-      <c r="AF37" s="86"/>
-      <c r="AG37" s="86"/>
-      <c r="AH37" s="86"/>
-      <c r="AI37" s="86"/>
-      <c r="AJ37" s="86"/>
-      <c r="AK37" s="86"/>
-      <c r="AL37" s="86"/>
-      <c r="AM37" s="86"/>
-      <c r="AN37" s="86"/>
-      <c r="AO37" s="86"/>
-      <c r="AP37" s="86"/>
-      <c r="AQ37" s="86"/>
-      <c r="AR37" s="86"/>
-      <c r="AS37" s="86"/>
+      <c r="K37" s="59"/>
+      <c r="L37" s="59"/>
+      <c r="M37" s="59"/>
+      <c r="N37" s="59"/>
+      <c r="O37" s="59"/>
+      <c r="P37" s="59"/>
+      <c r="Q37" s="59"/>
+      <c r="R37" s="59"/>
+      <c r="S37" s="59"/>
+      <c r="T37" s="59"/>
+      <c r="U37" s="59"/>
+      <c r="V37" s="59"/>
+      <c r="W37" s="59"/>
+      <c r="X37" s="59"/>
+      <c r="Y37" s="59"/>
+      <c r="Z37" s="59"/>
+      <c r="AA37" s="59"/>
+      <c r="AB37" s="59"/>
+      <c r="AC37" s="59"/>
+      <c r="AD37" s="59"/>
+      <c r="AE37" s="59"/>
+      <c r="AF37" s="59"/>
+      <c r="AG37" s="59"/>
+      <c r="AH37" s="59"/>
+      <c r="AI37" s="59"/>
+      <c r="AJ37" s="59"/>
+      <c r="AK37" s="59"/>
+      <c r="AL37" s="59"/>
+      <c r="AM37" s="59"/>
+      <c r="AN37" s="59"/>
+      <c r="AO37" s="59"/>
+      <c r="AP37" s="59"/>
+      <c r="AQ37" s="59"/>
+      <c r="AR37" s="59"/>
+      <c r="AS37" s="59"/>
     </row>
     <row r="38" spans="1:45" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="53"/>
@@ -3052,41 +3052,41 @@
       <c r="D38" s="19"/>
       <c r="E38" s="15"/>
       <c r="F38" s="15"/>
-      <c r="K38" s="86"/>
-      <c r="L38" s="86"/>
-      <c r="M38" s="86"/>
-      <c r="N38" s="86"/>
-      <c r="O38" s="86"/>
-      <c r="P38" s="86"/>
-      <c r="Q38" s="86"/>
-      <c r="R38" s="86"/>
-      <c r="S38" s="86"/>
-      <c r="T38" s="86"/>
-      <c r="U38" s="86"/>
-      <c r="V38" s="86"/>
-      <c r="W38" s="86"/>
-      <c r="X38" s="86"/>
-      <c r="Y38" s="86"/>
-      <c r="Z38" s="86"/>
-      <c r="AA38" s="86"/>
-      <c r="AB38" s="86"/>
-      <c r="AC38" s="86"/>
-      <c r="AD38" s="86"/>
-      <c r="AE38" s="86"/>
-      <c r="AF38" s="86"/>
-      <c r="AG38" s="86"/>
-      <c r="AH38" s="86"/>
-      <c r="AI38" s="86"/>
-      <c r="AJ38" s="86"/>
-      <c r="AK38" s="86"/>
-      <c r="AL38" s="86"/>
-      <c r="AM38" s="86"/>
-      <c r="AN38" s="86"/>
-      <c r="AO38" s="86"/>
-      <c r="AP38" s="86"/>
-      <c r="AQ38" s="86"/>
-      <c r="AR38" s="86"/>
-      <c r="AS38" s="86"/>
+      <c r="K38" s="59"/>
+      <c r="L38" s="59"/>
+      <c r="M38" s="59"/>
+      <c r="N38" s="59"/>
+      <c r="O38" s="59"/>
+      <c r="P38" s="59"/>
+      <c r="Q38" s="59"/>
+      <c r="R38" s="59"/>
+      <c r="S38" s="59"/>
+      <c r="T38" s="59"/>
+      <c r="U38" s="59"/>
+      <c r="V38" s="59"/>
+      <c r="W38" s="59"/>
+      <c r="X38" s="59"/>
+      <c r="Y38" s="59"/>
+      <c r="Z38" s="59"/>
+      <c r="AA38" s="59"/>
+      <c r="AB38" s="59"/>
+      <c r="AC38" s="59"/>
+      <c r="AD38" s="59"/>
+      <c r="AE38" s="59"/>
+      <c r="AF38" s="59"/>
+      <c r="AG38" s="59"/>
+      <c r="AH38" s="59"/>
+      <c r="AI38" s="59"/>
+      <c r="AJ38" s="59"/>
+      <c r="AK38" s="59"/>
+      <c r="AL38" s="59"/>
+      <c r="AM38" s="59"/>
+      <c r="AN38" s="59"/>
+      <c r="AO38" s="59"/>
+      <c r="AP38" s="59"/>
+      <c r="AQ38" s="59"/>
+      <c r="AR38" s="59"/>
+      <c r="AS38" s="59"/>
     </row>
     <row r="39" spans="1:45" ht="103" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="53"/>
@@ -3097,41 +3097,41 @@
       </c>
       <c r="E39" s="17"/>
       <c r="F39" s="17"/>
-      <c r="K39" s="86"/>
-      <c r="L39" s="86"/>
-      <c r="M39" s="86"/>
-      <c r="N39" s="86"/>
-      <c r="O39" s="86"/>
-      <c r="P39" s="86"/>
-      <c r="Q39" s="86"/>
-      <c r="R39" s="86"/>
-      <c r="S39" s="86"/>
-      <c r="T39" s="86"/>
-      <c r="U39" s="86"/>
-      <c r="V39" s="86"/>
-      <c r="W39" s="86"/>
-      <c r="X39" s="86"/>
-      <c r="Y39" s="86"/>
-      <c r="Z39" s="86"/>
-      <c r="AA39" s="86"/>
-      <c r="AB39" s="86"/>
-      <c r="AC39" s="86"/>
-      <c r="AD39" s="86"/>
-      <c r="AE39" s="86"/>
-      <c r="AF39" s="86"/>
-      <c r="AG39" s="86"/>
-      <c r="AH39" s="86"/>
-      <c r="AI39" s="86"/>
-      <c r="AJ39" s="86"/>
-      <c r="AK39" s="86"/>
-      <c r="AL39" s="86"/>
-      <c r="AM39" s="86"/>
-      <c r="AN39" s="86"/>
-      <c r="AO39" s="86"/>
-      <c r="AP39" s="86"/>
-      <c r="AQ39" s="86"/>
-      <c r="AR39" s="86"/>
-      <c r="AS39" s="86"/>
+      <c r="K39" s="59"/>
+      <c r="L39" s="59"/>
+      <c r="M39" s="59"/>
+      <c r="N39" s="59"/>
+      <c r="O39" s="59"/>
+      <c r="P39" s="59"/>
+      <c r="Q39" s="59"/>
+      <c r="R39" s="59"/>
+      <c r="S39" s="59"/>
+      <c r="T39" s="59"/>
+      <c r="U39" s="59"/>
+      <c r="V39" s="59"/>
+      <c r="W39" s="59"/>
+      <c r="X39" s="59"/>
+      <c r="Y39" s="59"/>
+      <c r="Z39" s="59"/>
+      <c r="AA39" s="59"/>
+      <c r="AB39" s="59"/>
+      <c r="AC39" s="59"/>
+      <c r="AD39" s="59"/>
+      <c r="AE39" s="59"/>
+      <c r="AF39" s="59"/>
+      <c r="AG39" s="59"/>
+      <c r="AH39" s="59"/>
+      <c r="AI39" s="59"/>
+      <c r="AJ39" s="59"/>
+      <c r="AK39" s="59"/>
+      <c r="AL39" s="59"/>
+      <c r="AM39" s="59"/>
+      <c r="AN39" s="59"/>
+      <c r="AO39" s="59"/>
+      <c r="AP39" s="59"/>
+      <c r="AQ39" s="59"/>
+      <c r="AR39" s="59"/>
+      <c r="AS39" s="59"/>
     </row>
     <row r="40" spans="1:45" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="53"/>
@@ -3147,19 +3147,19 @@
       <c r="C41" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="D41" s="73"/>
-      <c r="E41" s="74"/>
-      <c r="F41" s="75"/>
+      <c r="D41" s="63"/>
+      <c r="E41" s="64"/>
+      <c r="F41" s="65"/>
     </row>
     <row r="42" spans="1:45" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="53"/>
       <c r="B42" s="28"/>
       <c r="C42" s="44"/>
-      <c r="D42" s="71" t="s">
+      <c r="D42" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="E42" s="71"/>
-      <c r="F42" s="72"/>
+      <c r="E42" s="66"/>
+      <c r="F42" s="67"/>
     </row>
     <row r="43" spans="1:45" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="53"/>
@@ -3173,11 +3173,11 @@
       <c r="A44" s="53"/>
       <c r="B44" s="28"/>
       <c r="C44" s="44"/>
-      <c r="D44" s="71" t="s">
+      <c r="D44" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="E44" s="71"/>
-      <c r="F44" s="72"/>
+      <c r="E44" s="66"/>
+      <c r="F44" s="67"/>
     </row>
     <row r="45" spans="1:45" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="53"/>
@@ -3191,11 +3191,11 @@
       <c r="A46" s="53"/>
       <c r="B46" s="28"/>
       <c r="C46" s="44"/>
-      <c r="D46" s="71" t="s">
+      <c r="D46" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="E46" s="71"/>
-      <c r="F46" s="72"/>
+      <c r="E46" s="66"/>
+      <c r="F46" s="67"/>
     </row>
     <row r="47" spans="1:45" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="53"/>
@@ -3209,11 +3209,11 @@
       <c r="A48" s="53"/>
       <c r="B48" s="28"/>
       <c r="C48" s="44"/>
-      <c r="D48" s="71" t="s">
+      <c r="D48" s="66" t="s">
         <v>10</v>
       </c>
-      <c r="E48" s="71"/>
-      <c r="F48" s="72"/>
+      <c r="E48" s="66"/>
+      <c r="F48" s="67"/>
     </row>
     <row r="49" spans="1:6" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A49" s="53"/>
@@ -3229,19 +3229,19 @@
       <c r="C50" s="45" t="s">
         <v>19</v>
       </c>
-      <c r="D50" s="73"/>
-      <c r="E50" s="74"/>
-      <c r="F50" s="75"/>
+      <c r="D50" s="63"/>
+      <c r="E50" s="64"/>
+      <c r="F50" s="65"/>
     </row>
     <row r="51" spans="1:6" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A51" s="53"/>
       <c r="B51" s="28"/>
       <c r="C51" s="44"/>
-      <c r="D51" s="71" t="s">
+      <c r="D51" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="E51" s="71"/>
-      <c r="F51" s="72"/>
+      <c r="E51" s="66"/>
+      <c r="F51" s="67"/>
     </row>
     <row r="52" spans="1:6" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A52" s="53"/>
@@ -3255,11 +3255,11 @@
       <c r="A53" s="53"/>
       <c r="B53" s="28"/>
       <c r="C53" s="44"/>
-      <c r="D53" s="71" t="s">
+      <c r="D53" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="E53" s="71"/>
-      <c r="F53" s="72"/>
+      <c r="E53" s="66"/>
+      <c r="F53" s="67"/>
     </row>
     <row r="54" spans="1:6" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="53"/>
@@ -3273,11 +3273,11 @@
       <c r="A55" s="53"/>
       <c r="B55" s="28"/>
       <c r="C55" s="44"/>
-      <c r="D55" s="71" t="s">
+      <c r="D55" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="E55" s="71"/>
-      <c r="F55" s="72"/>
+      <c r="E55" s="66"/>
+      <c r="F55" s="67"/>
     </row>
     <row r="56" spans="1:6" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A56" s="53"/>
@@ -3291,11 +3291,11 @@
       <c r="A57" s="53"/>
       <c r="B57" s="28"/>
       <c r="C57" s="44"/>
-      <c r="D57" s="71" t="s">
+      <c r="D57" s="66" t="s">
         <v>10</v>
       </c>
-      <c r="E57" s="71"/>
-      <c r="F57" s="72"/>
+      <c r="E57" s="66"/>
+      <c r="F57" s="67"/>
     </row>
     <row r="58" spans="1:6" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="54"/>
@@ -3307,17 +3307,13 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="D32:F32"/>
-    <mergeCell ref="D41:F41"/>
-    <mergeCell ref="D50:F50"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="D53:F53"/>
-    <mergeCell ref="D57:F57"/>
-    <mergeCell ref="D48:F48"/>
-    <mergeCell ref="D46:F46"/>
-    <mergeCell ref="D42:F42"/>
-    <mergeCell ref="D44:F44"/>
-    <mergeCell ref="D55:F55"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="D18:D21"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="D14:F14"/>
     <mergeCell ref="E30:F30"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="E18:F18"/>
@@ -3327,13 +3323,17 @@
     <mergeCell ref="D23:D26"/>
     <mergeCell ref="D28:D31"/>
     <mergeCell ref="D22:F22"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="D18:D21"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="D57:F57"/>
+    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="D46:F46"/>
+    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="D44:F44"/>
+    <mergeCell ref="D55:F55"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="D41:F41"/>
+    <mergeCell ref="D50:F50"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="D53:F53"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>